<commit_message>
Rename market fields to Target/Live Markets; clarify the three meanings of scope
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01StVcJUwgS1Q5ccE9MpPikU
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -4169,7 +4169,7 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Target Markets / Scope</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Live Markets / Scope</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -13659,7 +13659,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Target Markets / Scope</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Live Markets / Scope</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -18163,6 +18163,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rename roadmap category to 'Close capability gaps' (migration 0010)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01StVcJUwgS1Q5ccE9MpPikU
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -880,12 +880,12 @@
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>New big bets · Grow customer revenues · Protect customer revenues · Operational efficiency · Close the gap with competitors</t>
+          <t>New big bets · Grow customer revenues · Protect customer revenues · Operational efficiency · Close capability gaps</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>New big bets, Grow customer revenues, Protect customer revenues, Operational efficiency, Close the gap with competitors</t>
+          <t>New big bets, Grow customer revenues, Protect customer revenues, Operational efficiency, Close capability gaps</t>
         </is>
       </c>
       <c r="H3" s="9" t="inlineStr">
@@ -19657,7 +19657,7 @@
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>Close the gap with competitors</t>
+          <t>Close capability gaps</t>
         </is>
       </c>
       <c r="M6" s="15" t="n"/>

</xml_diff>

<commit_message>
Build Status and Initiative Status: a closed ticket means the build is complete, not the initiative (0.12.0)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ERQpq8pxcAFVzGTKBxketD
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N166"/>
+  <dimension ref="A1:N167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -940,7 +940,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -11314,6 +11314,76 @@
         </is>
       </c>
       <c r="N166" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="9" t="inlineStr">
+        <is>
+          <t>N43</t>
+        </is>
+      </c>
+      <c r="B167" s="9" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C167" s="9" t="inlineStr">
+        <is>
+          <t>Initiative Status</t>
+        </is>
+      </c>
+      <c r="D167" s="9" t="inlineStr">
+        <is>
+          <t>initiative_status</t>
+        </is>
+      </c>
+      <c r="E167" s="9" t="inlineStr">
+        <is>
+          <t>Select</t>
+        </is>
+      </c>
+      <c r="F167" s="9" t="inlineStr">
+        <is>
+          <t>Backlog · Not Started · In Progress · Paused · Completed · Cancelled</t>
+        </is>
+      </c>
+      <c r="G167" s="9" t="inlineStr">
+        <is>
+          <t>Where the initiative itself stands, set by people (a closed GitHub or Jira ticket only means the build is complete: see Build Status).</t>
+        </is>
+      </c>
+      <c r="H167" s="9" t="inlineStr">
+        <is>
+          <t>Now where known</t>
+        </is>
+      </c>
+      <c r="I167" s="9" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J167" s="14" t="inlineStr">
+        <is>
+          <t>New (2026-10-23)</t>
+        </is>
+      </c>
+      <c r="K167" s="9" t="inlineStr">
+        <is>
+          <t>Split from Build Status (decided 2026-10-23): a closed GitHub or Jira ticket means the build is complete, not that the initiative is delivered, adopted and measured. People decide where the initiative stands.</t>
+        </is>
+      </c>
+      <c r="L167" s="9" t="inlineStr">
+        <is>
+          <t>Not synced. A closed linked ticket only sets Build Status and Build Completed; people decide where the initiative itself stands.</t>
+        </is>
+      </c>
+      <c r="M167" s="9" t="inlineStr">
+        <is>
+          <t>Column on items</t>
+        </is>
+      </c>
+      <c r="N167" s="9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11329,7 +11399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P169"/>
+  <dimension ref="A1:P170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11559,7 +11629,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -18174,15 +18244,61 @@
         <v>1</v>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>
-          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
-        </is>
+          <t>Initiative Status</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>initiative_status</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Select</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Editable</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P168" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="169">
       <c r="B169" t="inlineStr">
+        <is>
+          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" t="inlineStr">
         <is>
           <t>2026-10-23: the view columns (Prioritisation … History) on this sheet are SUPERSEDED by sheet 'Default views (ordered)' and docs/reference/default-views.csv (10 views, each with a reading order). Editing mode and the customer-safe flag on this sheet remain valid. 'In view count' is outdated.</t>
         </is>
@@ -19806,7 +19922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21085,7 +21201,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -21094,7 +21210,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -21108,12 +21224,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -21122,7 +21238,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
@@ -21136,21 +21252,21 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -21164,12 +21280,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Schedule Variance (pp)</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>schedule_variance_pp</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -21192,21 +21308,21 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Schedule Variance (pp)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>schedule_variance_pp</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -21220,12 +21336,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -21234,7 +21350,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -21248,21 +21364,21 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Blocked Issues (#)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>blocked_issues</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
@@ -21276,12 +21392,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Stale Issues (#)</t>
+          <t>Blocked Issues (#)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>stale_issues</t>
+          <t>blocked_issues</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -21304,12 +21420,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Scope Added (#)</t>
+          <t>Stale Issues (#)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>scope_added</t>
+          <t>stale_issues</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -21332,12 +21448,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Open PRs (#)</t>
+          <t>Scope Added (#)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>open_prs</t>
+          <t>scope_added</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -21360,12 +21476,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CI Status</t>
+          <t>Open PRs (#)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ci_status</t>
+          <t>open_prs</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -21388,12 +21504,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Assignees</t>
+          <t>CI Status</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>assignees</t>
+          <t>ci_status</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -21416,12 +21532,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Breakdown Status</t>
+          <t>Assignees</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>breakdown_status</t>
+          <t>assignees</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -21430,45 +21546,35 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Breakdown Status</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>breakdown_status</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>1</v>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="57">
@@ -21477,17 +21583,22 @@
           <t>Go-to-market</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+        </is>
+      </c>
       <c r="C57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -21511,16 +21622,16 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -21544,16 +21655,16 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -21563,6 +21674,11 @@
       </c>
       <c r="G59" t="n">
         <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -21572,21 +21688,21 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Audience</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G60" t="n">
@@ -21600,25 +21716,25 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Audience</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>audience</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -21628,16 +21744,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -21646,7 +21762,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
@@ -21656,16 +21772,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Date Precision</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>date_precision</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -21684,21 +21800,21 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Target Markets</t>
+          <t>Date Precision</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>target_scope</t>
+          <t>date_precision</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G64" t="n">
@@ -21712,16 +21828,16 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Live Markets</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>live_scope</t>
+          <t>target_scope</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -21740,21 +21856,21 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Target Segments (customer-safe)</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>target_segments</t>
+          <t>live_scope</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G66" t="n">
@@ -21768,21 +21884,21 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Target Customers (#)</t>
+          <t>Target Segments (customer-safe)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>target_customers</t>
+          <t>target_segments</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G67" t="n">
@@ -21796,16 +21912,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Customers Live (#)</t>
+          <t>Target Customers (#)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>customers_live</t>
+          <t>target_customers</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -21814,7 +21930,7 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -21824,16 +21940,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Roll-out %</t>
+          <t>Customers Live (#)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>rollout_pct</t>
+          <t>customers_live</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -21852,16 +21968,16 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Roll-out %</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>rollout_pct</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -21880,25 +21996,25 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Value Proposition (customer-safe)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>value_proposition</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G71" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72">
@@ -21908,16 +22024,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Value Proposition (customer-safe)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>value_proposition</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -21936,21 +22052,21 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>GTM / Enablement Notes</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>gtm_enablement_notes</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G73" t="n">
@@ -21964,21 +22080,21 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Screenshots</t>
+          <t>GTM / Enablement Notes</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>screenshots</t>
+          <t>gtm_enablement_notes</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G74" t="n">
@@ -21988,25 +22104,20 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Outcomes</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Screenshots</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>screenshots</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -22016,11 +22127,6 @@
       </c>
       <c r="G75" t="n">
         <v>1</v>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="76">
@@ -22029,17 +22135,22 @@
           <t>Outcomes</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+        </is>
+      </c>
       <c r="C76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -22063,16 +22174,16 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -22096,16 +22207,16 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -22115,6 +22226,11 @@
       </c>
       <c r="G78" t="n">
         <v>1</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -22124,25 +22240,25 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Outcome Status</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>outcome_status</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G79" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -22152,16 +22268,16 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Outcome Review Date</t>
+          <t>Outcome Status</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>outcome_review_date</t>
+          <t>outcome_status</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -22180,25 +22296,25 @@
         </is>
       </c>
       <c r="C81" t="n">
+        <v>6</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Outcome Review Date</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>outcome_review_date</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Outcomes</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
         <v>7</v>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Primary KR (Metric Name)</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>kr_metric</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="G81" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -22208,16 +22324,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Primary KR Unit</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>kr_unit</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -22236,16 +22352,16 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Primary KR Start Value</t>
+          <t>Primary KR Unit</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>kr_start</t>
+          <t>kr_unit</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -22264,16 +22380,16 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR Start Value</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_start</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -22292,25 +22408,25 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Realized KR Value</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>realized_kr_value</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G85" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -22320,16 +22436,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>% Realized KR Value</t>
+          <t>Realized KR Value</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>kr_realized_pct</t>
+          <t>realized_kr_value</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -22348,21 +22464,21 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>% Realized KR Value</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>kr_realized_pct</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G87" t="n">
@@ -22376,25 +22492,25 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G88" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="89">
@@ -22404,25 +22520,25 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Realized EUR per year</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>realized_per_year</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -22432,16 +22548,16 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Value vs Prediction (%)</t>
+          <t>Realized EUR per year</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>value_variance_pct</t>
+          <t>realized_per_year</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -22460,16 +22576,16 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Outcome Verdict</t>
+          <t>Value vs Prediction (%)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>outcome_verdict</t>
+          <t>value_variance_pct</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -22488,16 +22604,16 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Time to First Use (days)</t>
+          <t>Outcome Verdict</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>time_to_first_use_days</t>
+          <t>outcome_verdict</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -22516,16 +22632,16 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Retention (%)</t>
+          <t>Time to First Use (days)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>retention_pct</t>
+          <t>time_to_first_use_days</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -22544,16 +22660,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Retention (%)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>retention_pct</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -22568,39 +22684,29 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Leadership</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G95" t="n">
-        <v>1</v>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="96">
@@ -22609,17 +22715,22 @@
           <t>Leadership</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+        </is>
+      </c>
       <c r="C96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -22643,16 +22754,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -22676,16 +22787,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -22695,6 +22806,11 @@
       </c>
       <c r="G98" t="n">
         <v>1</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -22704,16 +22820,16 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Initiative Group</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -22732,16 +22848,16 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Roadmap Category</t>
+          <t>Initiative Group</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>roadmap_category</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -22760,16 +22876,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Roadmap Category</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>roadmap_category</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -22788,16 +22904,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -22816,25 +22932,25 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G103" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -22844,25 +22960,25 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G104" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
@@ -22872,16 +22988,16 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -22900,25 +23016,25 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
@@ -22928,16 +23044,16 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -22956,21 +23072,21 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G108" t="n">
@@ -22984,25 +23100,25 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Current Gate</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>current_gate</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Gates</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
@@ -23012,25 +23128,25 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Current Gate</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>current_gate</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Gates</t>
         </is>
       </c>
       <c r="G110" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="111">
@@ -23040,25 +23156,25 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>sponsor</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G111" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112">
@@ -23068,21 +23184,21 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Next Review Date</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>next_review_date</t>
+          <t>sponsor</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G112" t="n">
@@ -23096,21 +23212,21 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Next Review Date</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>next_review_date</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G113" t="n">
@@ -23120,25 +23236,20 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Discovery</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -23148,11 +23259,6 @@
       </c>
       <c r="G114" t="n">
         <v>1</v>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="115">
@@ -23161,17 +23267,22 @@
           <t>Discovery</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+        </is>
+      </c>
       <c r="C115" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -23195,16 +23306,16 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -23228,16 +23339,16 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -23247,6 +23358,11 @@
       </c>
       <c r="G117" t="n">
         <v>1</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -23256,16 +23372,16 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Change Type</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>change_type</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -23284,16 +23400,16 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
+          <t>Change Type</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>hypothesis</t>
+          <t>change_type</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -23312,21 +23428,21 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Request Origin</t>
+          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>request_origin</t>
+          <t>hypothesis</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G120" t="n">
@@ -23340,16 +23456,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Customers Requesting (#)</t>
+          <t>Request Origin</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>customers_requesting</t>
+          <t>request_origin</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -23368,21 +23484,21 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Customers Requesting (#)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>customers_requesting</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G122" t="n">
@@ -23396,21 +23512,21 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Cost of Not Doing (strategic risk)</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>cost_of_not_doing</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G123" t="n">
@@ -23424,16 +23540,16 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Related / Overlaps With (Initiative IDs)</t>
+          <t>Cost of Not Doing (strategic risk)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>related_to</t>
+          <t>cost_of_not_doing</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -23452,16 +23568,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Dependencies / Blockers</t>
+          <t>Related / Overlaps With (Initiative IDs)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>dependencies_blockers</t>
+          <t>related_to</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -23480,16 +23596,16 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Dependencies / Blockers</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>dependencies_blockers</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -23508,16 +23624,16 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Value Type</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>value_basis</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -23536,16 +23652,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Time to First Revenue (months)</t>
+          <t>Value Basis</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>time_to_first_revenue_months</t>
+          <t>value_basis</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -23564,16 +23680,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Primary KR (Metric Name)</t>
+          <t>Time to First Revenue (months)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>kr_metric</t>
+          <t>time_to_first_revenue_months</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -23592,16 +23708,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -23620,21 +23736,21 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Artifacts (links)</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>artifacts</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G131" t="n">
@@ -23648,25 +23764,25 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Artifacts (links)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>artifacts</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G132" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133">
@@ -23676,16 +23792,16 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Spec Status</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>spec_status</t>
+          <t>documents</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -23704,25 +23820,25 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Spec Status</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>product_manager</t>
+          <t>spec_status</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G134" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="135">
@@ -23732,16 +23848,16 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>designer</t>
+          <t>product_manager</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -23760,16 +23876,16 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>designer</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -23788,16 +23904,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Business Manager</t>
+          <t>Analyst</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>business_manager</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -23816,21 +23932,21 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>AI Draft (needs review)</t>
+          <t>Business Manager</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>ai_draft</t>
+          <t>business_manager</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G138" t="n">
@@ -23840,39 +23956,29 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Timeline</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+          <t>Discovery</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>AI Draft (needs review)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>ai_draft</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G139" t="n">
         <v>1</v>
-      </c>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="140">
@@ -23881,17 +23987,22 @@
           <t>Timeline</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+        </is>
+      </c>
       <c r="C140" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -23915,16 +24026,16 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -23948,16 +24059,16 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -23967,6 +24078,11 @@
       </c>
       <c r="G142" t="n">
         <v>1</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="143">
@@ -23976,25 +24092,25 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Days in Current Phase</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>days_in_phase</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G143" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144">
@@ -24004,25 +24120,25 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Days in Current Phase</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>days_in_phase</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G144" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
@@ -24032,16 +24148,16 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Start Discovery</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>start_discovery</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -24060,16 +24176,16 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Start Definition</t>
+          <t>Start Discovery</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>start_definition</t>
+          <t>start_discovery</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -24088,16 +24204,16 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Start Building</t>
+          <t>Start Definition</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>start_building</t>
+          <t>start_definition</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -24116,16 +24232,16 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Start Beta-Test</t>
+          <t>Start Building</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>start_beta</t>
+          <t>start_building</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -24144,16 +24260,16 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Start Experiment</t>
+          <t>Start Beta-Test</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>start_experiment</t>
+          <t>start_beta</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -24172,16 +24288,16 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Start Roll-Out</t>
+          <t>Start Experiment</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>start_rollout</t>
+          <t>start_experiment</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -24200,16 +24316,16 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>G2M Date (actual)</t>
+          <t>Start Roll-Out</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>g2m_date_actual</t>
+          <t>start_rollout</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -24228,25 +24344,25 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Discovery Time (days)</t>
+          <t>G2M Date (actual)</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>time_discovery_days</t>
+          <t>g2m_date_actual</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G152" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="153">
@@ -24256,16 +24372,16 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Definition Time (days)</t>
+          <t>Discovery Time (days)</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>time_definition_days</t>
+          <t>time_discovery_days</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -24284,16 +24400,16 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Building Time (days)</t>
+          <t>Definition Time (days)</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>time_building_days</t>
+          <t>time_definition_days</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -24312,16 +24428,16 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Beta-Test Time (days)</t>
+          <t>Building Time (days)</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>time_beta_days</t>
+          <t>time_building_days</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -24340,16 +24456,16 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Experiment Time (days)</t>
+          <t>Beta-Test Time (days)</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>time_experiment_days</t>
+          <t>time_beta_days</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -24368,16 +24484,16 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Roll-Out Time (days)</t>
+          <t>Experiment Time (days)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>time_rollout_days</t>
+          <t>time_experiment_days</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -24396,16 +24512,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Time to Market (days)</t>
+          <t>Roll-Out Time (days)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>time_to_market_days</t>
+          <t>time_rollout_days</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -24424,16 +24540,16 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Actual Build (weeks)</t>
+          <t>Time to Market (days)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>actual_build_weeks</t>
+          <t>time_to_market_days</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -24452,16 +24568,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Build vs Estimate High (%)</t>
+          <t>Actual Build (weeks)</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>build_vs_estimate_high_pct</t>
+          <t>actual_build_weeks</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -24480,16 +24596,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Blocked Days</t>
+          <t>Build vs Estimate High (%)</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>blocked_days</t>
+          <t>build_vs_estimate_high_pct</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -24504,39 +24620,29 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>History</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Blocked Days</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>blocked_days</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G162" t="n">
-        <v>1</v>
-      </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="163">
@@ -24545,17 +24651,22 @@
           <t>History</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+        </is>
+      </c>
       <c r="C163" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -24579,16 +24690,16 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -24612,16 +24723,16 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -24630,7 +24741,12 @@
         </is>
       </c>
       <c r="G165" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="166">
@@ -24640,16 +24756,16 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -24668,16 +24784,16 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -24686,7 +24802,7 @@
         </is>
       </c>
       <c r="G167" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168">
@@ -24696,21 +24812,21 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G168" t="n">
@@ -24724,21 +24840,21 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Decided By</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>decided_by</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G169" t="n">
@@ -24752,16 +24868,16 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Decision Date</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>decision_date</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -24780,21 +24896,21 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Status Changed At</t>
+          <t>Decided By</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>status_changed_at</t>
+          <t>decided_by</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G171" t="n">
@@ -24808,21 +24924,21 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Phase Changed At</t>
+          <t>Decision Date</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>phase_changed_at</t>
+          <t>decision_date</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G172" t="n">
@@ -24836,21 +24952,21 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>Status Changed At</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>last_edited_at</t>
+          <t>status_changed_at</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G173" t="n">
@@ -24864,16 +24980,16 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Last Edited By</t>
+          <t>Phase Changed At</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>last_edited_by</t>
+          <t>phase_changed_at</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -24892,21 +25008,21 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Created At</t>
+          <t>Last Updated</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>last_edited_at</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G175" t="n">
@@ -24920,16 +25036,16 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Created By</t>
+          <t>Last Edited By</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>last_edited_by</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -24948,16 +25064,16 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Created Via</t>
+          <t>Created At</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>created_via</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -24976,16 +25092,16 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Last Reviewed</t>
+          <t>Created By</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>last_reviewed_at</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -25004,16 +25120,16 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Review Overdue</t>
+          <t>Created Via</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>review_overdue</t>
+          <t>created_via</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -25022,7 +25138,7 @@
         </is>
       </c>
       <c r="G179" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="180">
@@ -25032,16 +25148,16 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Item Age (days)</t>
+          <t>Last Reviewed</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>item_age_days</t>
+          <t>last_reviewed_at</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -25050,7 +25166,7 @@
         </is>
       </c>
       <c r="G180" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="181">
@@ -25060,16 +25176,16 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Archived</t>
+          <t>Review Overdue</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>review_overdue</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -25078,78 +25194,63 @@
         </is>
       </c>
       <c r="G181" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Cycle review</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Item Age (days)</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_age_days</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G182" t="n">
-        <v>1</v>
-      </c>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Cycle review</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>archived</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G183" t="n">
         <v>1</v>
-      </c>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="184">
@@ -25158,17 +25259,22 @@
           <t>Cycle review</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+        </is>
+      </c>
       <c r="C184" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -25192,16 +25298,16 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -25211,6 +25317,11 @@
       </c>
       <c r="G185" t="n">
         <v>1</v>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="186">
@@ -25220,25 +25331,30 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G186" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="187">
@@ -25248,25 +25364,25 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G187" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -25276,16 +25392,16 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Candidate Tag</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>candidate_tag</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -25304,16 +25420,16 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Deferred Count</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>deferred_count</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -25332,16 +25448,16 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Deferral Reason</t>
+          <t>Candidate Tag</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>deferral_reason</t>
+          <t>candidate_tag</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -25360,16 +25476,16 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Added After Commit</t>
+          <t>Deferred Count</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>added_after_commit</t>
+          <t>deferred_count</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -25388,25 +25504,25 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Deferral Reason</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>deferral_reason</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G192" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="193">
@@ -25416,25 +25532,25 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Added After Commit</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>added_after_commit</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G193" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="194">
@@ -25444,25 +25560,25 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G194" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -25472,16 +25588,16 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>MoSCoW</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>moscow</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -25500,24 +25616,80 @@
         </is>
       </c>
       <c r="C196" t="n">
+        <v>13</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Fit by Team</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>fit_by_team</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G196" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>14</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>MoSCoW</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>moscow</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G197" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
         <v>15</v>
       </c>
-      <c r="D196" t="inlineStr">
+      <c r="D198" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr">
+      <c r="E198" t="inlineStr">
         <is>
           <t>decision</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr">
+      <c r="F198" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="G196" t="n">
+      <c r="G198" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Issue number next to the Initiative ID and a Markdown Description field (0.24.0)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RLE7CotBaUe74bPtiiRYNc
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N167"/>
+  <dimension ref="A1:N168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11387,6 +11387,72 @@
         <v>1</v>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" s="9" t="inlineStr">
+        <is>
+          <t>N44</t>
+        </is>
+      </c>
+      <c r="B168" s="9" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D168" s="9" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E168" s="9" t="inlineStr">
+        <is>
+          <t>Long text</t>
+        </is>
+      </c>
+      <c r="F168" s="9" t="n"/>
+      <c r="G168" s="9" t="inlineStr">
+        <is>
+          <t>The technical description that engineers and agents work from, written in Markdown (headings, lists, links, tables). It becomes its own section of the tracking issue. It is visible to everyone who can see the issue, so keep value, customers and decisions out of it.</t>
+        </is>
+      </c>
+      <c r="H168" s="9" t="inlineStr">
+        <is>
+          <t>Before the push</t>
+        </is>
+      </c>
+      <c r="I168" s="9" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J168" s="14" t="inlineStr">
+        <is>
+          <t>New (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="K168" s="9" t="inlineStr">
+        <is>
+          <t>Asked for in the orchestration spec (Ashu, 2026-10-26): the place where the AI agent drafts and refines what is to be built. Markdown is stored; text is sanitised before it leaves the app.</t>
+        </is>
+      </c>
+      <c r="L168" s="9" t="inlineStr">
+        <is>
+          <t>App -&gt; GitHub: own section 'Description' of the managed block of the issue body (Markdown). Do not put value, customers or decisions in it.</t>
+        </is>
+      </c>
+      <c r="M168" s="9" t="inlineStr">
+        <is>
+          <t>Column on items</t>
+        </is>
+      </c>
+      <c r="N168" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11399,7 +11465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P170"/>
+  <dimension ref="A1:P171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18293,12 +18359,39 @@
     <row r="169">
       <c r="B169" t="inlineStr">
         <is>
-          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Long text</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Editable</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="B170" t="inlineStr">
+        <is>
+          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" t="inlineStr">
         <is>
           <t>2026-10-23: the view columns (Prioritisation … History) on this sheet are SUPERSEDED by sheet 'Default views (ordered)' and docs/reference/default-views.csv (10 views, each with a reading order). Editing mode and the customer-safe flag on this sheet remain valid. 'In view count' is outdated.</t>
         </is>
@@ -18425,7 +18518,7 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Summary, Hypothesis, Artifacts, backlink</t>
+          <t>Summary, Description, Hypothesis, Artifacts, backlink</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -18445,7 +18538,7 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Text outside the markers is never touched. Do not put value, customers or decisions in the body (repos can be public).</t>
+          <t>Text outside the markers is never touched. Do not put value, customers or decisions in the body (repos can be public). Description is Markdown and is its own section of the block.</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
@@ -19922,7 +20015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21224,12 +21317,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Build Status</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>description</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -21238,7 +21331,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -21252,12 +21345,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -21266,7 +21359,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46">
@@ -21280,21 +21373,21 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -21308,12 +21401,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Schedule Variance (pp)</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>schedule_variance_pp</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -21336,21 +21429,21 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Schedule Variance (pp)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>schedule_variance_pp</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
@@ -21364,12 +21457,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -21378,7 +21471,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -21392,21 +21485,21 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Blocked Issues (#)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>blocked_issues</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -21420,12 +21513,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Stale Issues (#)</t>
+          <t>Blocked Issues (#)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>stale_issues</t>
+          <t>blocked_issues</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -21448,12 +21541,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Scope Added (#)</t>
+          <t>Stale Issues (#)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>scope_added</t>
+          <t>stale_issues</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -21476,12 +21569,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Open PRs (#)</t>
+          <t>Scope Added (#)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>open_prs</t>
+          <t>scope_added</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -21504,12 +21597,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CI Status</t>
+          <t>Open PRs (#)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ci_status</t>
+          <t>open_prs</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -21532,12 +21625,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Assignees</t>
+          <t>CI Status</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>assignees</t>
+          <t>ci_status</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -21560,12 +21653,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Breakdown Status</t>
+          <t>Assignees</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>breakdown_status</t>
+          <t>assignees</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -21574,45 +21667,35 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Breakdown Status</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>breakdown_status</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G57" t="n">
-        <v>1</v>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="58">
@@ -21621,17 +21704,22 @@
           <t>Go-to-market</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+        </is>
+      </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -21655,16 +21743,16 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -21688,16 +21776,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -21707,6 +21795,11 @@
       </c>
       <c r="G60" t="n">
         <v>1</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -21716,21 +21809,21 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Audience</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G61" t="n">
@@ -21744,25 +21837,25 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Audience</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>audience</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -21772,16 +21865,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -21790,7 +21883,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -21800,16 +21893,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Date Precision</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>date_precision</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -21828,21 +21921,21 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Target Markets</t>
+          <t>Date Precision</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>target_scope</t>
+          <t>date_precision</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G65" t="n">
@@ -21856,16 +21949,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Live Markets</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>live_scope</t>
+          <t>target_scope</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -21884,21 +21977,21 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Target Segments (customer-safe)</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>target_segments</t>
+          <t>live_scope</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G67" t="n">
@@ -21912,21 +22005,21 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Target Customers (#)</t>
+          <t>Target Segments (customer-safe)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>target_customers</t>
+          <t>target_segments</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -21940,16 +22033,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Customers Live (#)</t>
+          <t>Target Customers (#)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>customers_live</t>
+          <t>target_customers</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -21958,7 +22051,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -21968,16 +22061,16 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Roll-out %</t>
+          <t>Customers Live (#)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>rollout_pct</t>
+          <t>customers_live</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -21996,16 +22089,16 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Roll-out %</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>rollout_pct</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -22024,25 +22117,25 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Value Proposition (customer-safe)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>value_proposition</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G72" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73">
@@ -22052,16 +22145,16 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Value Proposition (customer-safe)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>value_proposition</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -22080,21 +22173,21 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>GTM / Enablement Notes</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>gtm_enablement_notes</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G74" t="n">
@@ -22108,21 +22201,21 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Screenshots</t>
+          <t>GTM / Enablement Notes</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>screenshots</t>
+          <t>gtm_enablement_notes</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G75" t="n">
@@ -22132,25 +22225,20 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Outcomes</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Screenshots</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>screenshots</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -22160,11 +22248,6 @@
       </c>
       <c r="G76" t="n">
         <v>1</v>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="77">
@@ -22173,17 +22256,22 @@
           <t>Outcomes</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+        </is>
+      </c>
       <c r="C77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -22207,16 +22295,16 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -22240,16 +22328,16 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -22259,6 +22347,11 @@
       </c>
       <c r="G79" t="n">
         <v>1</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -22268,25 +22361,25 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Outcome Status</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>outcome_status</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G80" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -22296,16 +22389,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Outcome Review Date</t>
+          <t>Outcome Status</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>outcome_review_date</t>
+          <t>outcome_status</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -22324,25 +22417,25 @@
         </is>
       </c>
       <c r="C82" t="n">
+        <v>6</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Outcome Review Date</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>outcome_review_date</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Outcomes</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
         <v>7</v>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Primary KR (Metric Name)</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>kr_metric</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="G82" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -22352,16 +22445,16 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Primary KR Unit</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>kr_unit</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -22380,16 +22473,16 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Primary KR Start Value</t>
+          <t>Primary KR Unit</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>kr_start</t>
+          <t>kr_unit</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -22408,16 +22501,16 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR Start Value</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_start</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -22436,25 +22529,25 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Realized KR Value</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>realized_kr_value</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G86" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -22464,16 +22557,16 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>% Realized KR Value</t>
+          <t>Realized KR Value</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>kr_realized_pct</t>
+          <t>realized_kr_value</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -22492,21 +22585,21 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>% Realized KR Value</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>kr_realized_pct</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G88" t="n">
@@ -22520,25 +22613,25 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90">
@@ -22548,25 +22641,25 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Realized EUR per year</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>realized_per_year</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G90" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -22576,16 +22669,16 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Value vs Prediction (%)</t>
+          <t>Realized EUR per year</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>value_variance_pct</t>
+          <t>realized_per_year</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -22604,16 +22697,16 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Outcome Verdict</t>
+          <t>Value vs Prediction (%)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>outcome_verdict</t>
+          <t>value_variance_pct</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -22632,16 +22725,16 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Time to First Use (days)</t>
+          <t>Outcome Verdict</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>time_to_first_use_days</t>
+          <t>outcome_verdict</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -22660,16 +22753,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Retention (%)</t>
+          <t>Time to First Use (days)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>retention_pct</t>
+          <t>time_to_first_use_days</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -22688,16 +22781,16 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Retention (%)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>retention_pct</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -22712,39 +22805,29 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Leadership</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G96" t="n">
-        <v>1</v>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="97">
@@ -22753,17 +22836,22 @@
           <t>Leadership</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+        </is>
+      </c>
       <c r="C97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -22787,16 +22875,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -22820,16 +22908,16 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -22839,6 +22927,11 @@
       </c>
       <c r="G99" t="n">
         <v>1</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -22848,16 +22941,16 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Initiative Group</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -22876,16 +22969,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Roadmap Category</t>
+          <t>Initiative Group</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>roadmap_category</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -22904,16 +22997,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Roadmap Category</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>roadmap_category</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -22932,16 +23025,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -22960,25 +23053,25 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G104" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -22988,25 +23081,25 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G105" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="106">
@@ -23016,16 +23109,16 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -23044,25 +23137,25 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
@@ -23072,16 +23165,16 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -23100,21 +23193,21 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G109" t="n">
@@ -23128,25 +23221,25 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Current Gate</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>current_gate</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Gates</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G110" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -23156,25 +23249,25 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Current Gate</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>current_gate</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Gates</t>
         </is>
       </c>
       <c r="G111" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="112">
@@ -23184,25 +23277,25 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>sponsor</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G112" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113">
@@ -23212,21 +23305,21 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Next Review Date</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>next_review_date</t>
+          <t>sponsor</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G113" t="n">
@@ -23240,21 +23333,21 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Next Review Date</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>next_review_date</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G114" t="n">
@@ -23264,25 +23357,20 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Discovery</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -23292,11 +23380,6 @@
       </c>
       <c r="G115" t="n">
         <v>1</v>
-      </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="116">
@@ -23305,17 +23388,22 @@
           <t>Discovery</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+        </is>
+      </c>
       <c r="C116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -23339,16 +23427,16 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -23372,16 +23460,16 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -23391,6 +23479,11 @@
       </c>
       <c r="G118" t="n">
         <v>1</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -23400,16 +23493,16 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Change Type</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>change_type</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -23428,16 +23521,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
+          <t>Change Type</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>hypothesis</t>
+          <t>change_type</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -23456,21 +23549,21 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Request Origin</t>
+          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>request_origin</t>
+          <t>hypothesis</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G121" t="n">
@@ -23484,16 +23577,16 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Customers Requesting (#)</t>
+          <t>Request Origin</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>customers_requesting</t>
+          <t>request_origin</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -23512,21 +23605,21 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Customers Requesting (#)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>customers_requesting</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G123" t="n">
@@ -23540,21 +23633,21 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Cost of Not Doing (strategic risk)</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>cost_of_not_doing</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -23568,16 +23661,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Related / Overlaps With (Initiative IDs)</t>
+          <t>Cost of Not Doing (strategic risk)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>related_to</t>
+          <t>cost_of_not_doing</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -23596,16 +23689,16 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Dependencies / Blockers</t>
+          <t>Related / Overlaps With (Initiative IDs)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>dependencies_blockers</t>
+          <t>related_to</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -23624,16 +23717,16 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Dependencies / Blockers</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>dependencies_blockers</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -23652,16 +23745,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Value Type</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>value_basis</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -23680,16 +23773,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Time to First Revenue (months)</t>
+          <t>Value Basis</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>time_to_first_revenue_months</t>
+          <t>value_basis</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -23708,16 +23801,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Primary KR (Metric Name)</t>
+          <t>Time to First Revenue (months)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>kr_metric</t>
+          <t>time_to_first_revenue_months</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -23736,16 +23829,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -23764,21 +23857,21 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Artifacts (links)</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>artifacts</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G132" t="n">
@@ -23792,25 +23885,25 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Artifacts (links)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>artifacts</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G133" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -23820,16 +23913,16 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Spec Status</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>spec_status</t>
+          <t>documents</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -23848,25 +23941,25 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Spec Status</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>product_manager</t>
+          <t>spec_status</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G135" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="136">
@@ -23876,16 +23969,16 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>designer</t>
+          <t>product_manager</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -23904,16 +23997,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>designer</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -23932,16 +24025,16 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Business Manager</t>
+          <t>Analyst</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>business_manager</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -23960,21 +24053,21 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>AI Draft (needs review)</t>
+          <t>Business Manager</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>ai_draft</t>
+          <t>business_manager</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G139" t="n">
@@ -23984,39 +24077,29 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Timeline</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+          <t>Discovery</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>AI Draft (needs review)</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>ai_draft</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G140" t="n">
         <v>1</v>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="141">
@@ -24025,17 +24108,22 @@
           <t>Timeline</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+        </is>
+      </c>
       <c r="C141" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -24059,16 +24147,16 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -24092,16 +24180,16 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -24111,6 +24199,11 @@
       </c>
       <c r="G143" t="n">
         <v>1</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="144">
@@ -24120,25 +24213,25 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Days in Current Phase</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>days_in_phase</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="145">
@@ -24148,25 +24241,25 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Days in Current Phase</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>days_in_phase</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G145" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="146">
@@ -24176,16 +24269,16 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Start Discovery</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>start_discovery</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -24204,16 +24297,16 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Start Definition</t>
+          <t>Start Discovery</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>start_definition</t>
+          <t>start_discovery</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -24232,16 +24325,16 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Start Building</t>
+          <t>Start Definition</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>start_building</t>
+          <t>start_definition</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -24260,16 +24353,16 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Start Beta-Test</t>
+          <t>Start Building</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>start_beta</t>
+          <t>start_building</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -24288,16 +24381,16 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Start Experiment</t>
+          <t>Start Beta-Test</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>start_experiment</t>
+          <t>start_beta</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -24316,16 +24409,16 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Start Roll-Out</t>
+          <t>Start Experiment</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>start_rollout</t>
+          <t>start_experiment</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -24344,16 +24437,16 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>G2M Date (actual)</t>
+          <t>Start Roll-Out</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>g2m_date_actual</t>
+          <t>start_rollout</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -24372,25 +24465,25 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Discovery Time (days)</t>
+          <t>G2M Date (actual)</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>time_discovery_days</t>
+          <t>g2m_date_actual</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G153" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="154">
@@ -24400,16 +24493,16 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Definition Time (days)</t>
+          <t>Discovery Time (days)</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>time_definition_days</t>
+          <t>time_discovery_days</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -24428,16 +24521,16 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Building Time (days)</t>
+          <t>Definition Time (days)</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>time_building_days</t>
+          <t>time_definition_days</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -24456,16 +24549,16 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Beta-Test Time (days)</t>
+          <t>Building Time (days)</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>time_beta_days</t>
+          <t>time_building_days</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -24484,16 +24577,16 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Experiment Time (days)</t>
+          <t>Beta-Test Time (days)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>time_experiment_days</t>
+          <t>time_beta_days</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -24512,16 +24605,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Roll-Out Time (days)</t>
+          <t>Experiment Time (days)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>time_rollout_days</t>
+          <t>time_experiment_days</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -24540,16 +24633,16 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Time to Market (days)</t>
+          <t>Roll-Out Time (days)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>time_to_market_days</t>
+          <t>time_rollout_days</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -24568,16 +24661,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Actual Build (weeks)</t>
+          <t>Time to Market (days)</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>actual_build_weeks</t>
+          <t>time_to_market_days</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -24596,16 +24689,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Build vs Estimate High (%)</t>
+          <t>Actual Build (weeks)</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>build_vs_estimate_high_pct</t>
+          <t>actual_build_weeks</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -24624,16 +24717,16 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Blocked Days</t>
+          <t>Build vs Estimate High (%)</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>blocked_days</t>
+          <t>build_vs_estimate_high_pct</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -24648,39 +24741,29 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>History</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Blocked Days</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>blocked_days</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G163" t="n">
-        <v>1</v>
-      </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="164">
@@ -24689,17 +24772,22 @@
           <t>History</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+        </is>
+      </c>
       <c r="C164" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -24723,16 +24811,16 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -24756,16 +24844,16 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>initiative_status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -24775,6 +24863,11 @@
       </c>
       <c r="G166" t="n">
         <v>1</v>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="167">
@@ -24784,16 +24877,16 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Build Status</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -24802,7 +24895,7 @@
         </is>
       </c>
       <c r="G167" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="168">
@@ -24812,16 +24905,16 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -24830,7 +24923,7 @@
         </is>
       </c>
       <c r="G168" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169">
@@ -24840,16 +24933,16 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -24868,21 +24961,21 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G170" t="n">
@@ -24896,16 +24989,16 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Decided By</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>decided_by</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -24924,16 +25017,16 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Decision Date</t>
+          <t>Decided By</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>decision_date</t>
+          <t>decided_by</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -24952,21 +25045,21 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Status Changed At</t>
+          <t>Decision Date</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>status_changed_at</t>
+          <t>decision_date</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G173" t="n">
@@ -24980,16 +25073,16 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Phase Changed At</t>
+          <t>Status Changed At</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>phase_changed_at</t>
+          <t>status_changed_at</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -25008,21 +25101,21 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>Phase Changed At</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>last_edited_at</t>
+          <t>phase_changed_at</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G175" t="n">
@@ -25036,21 +25129,21 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Last Edited By</t>
+          <t>Last Updated</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>last_edited_by</t>
+          <t>last_edited_at</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G176" t="n">
@@ -25064,16 +25157,16 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Created At</t>
+          <t>Last Edited By</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>last_edited_by</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -25092,16 +25185,16 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Created By</t>
+          <t>Created At</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -25120,16 +25213,16 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Created Via</t>
+          <t>Created By</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>created_via</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -25148,16 +25241,16 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Last Reviewed</t>
+          <t>Created Via</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>last_reviewed_at</t>
+          <t>created_via</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -25176,16 +25269,16 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Review Overdue</t>
+          <t>Last Reviewed</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>review_overdue</t>
+          <t>last_reviewed_at</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -25194,7 +25287,7 @@
         </is>
       </c>
       <c r="G181" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -25204,16 +25297,16 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Item Age (days)</t>
+          <t>Review Overdue</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>item_age_days</t>
+          <t>review_overdue</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -25232,16 +25325,16 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Archived</t>
+          <t>Item Age (days)</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>item_age_days</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -25250,45 +25343,35 @@
         </is>
       </c>
       <c r="G183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Cycle review</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>archived</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G184" t="n">
         <v>1</v>
-      </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="185">
@@ -25297,17 +25380,22 @@
           <t>Cycle review</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+        </is>
+      </c>
       <c r="C185" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -25331,16 +25419,16 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -25364,16 +25452,16 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -25383,6 +25471,11 @@
       </c>
       <c r="G187" t="n">
         <v>1</v>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="188">
@@ -25392,25 +25485,25 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G188" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="189">
@@ -25420,16 +25513,16 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -25448,16 +25541,16 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Candidate Tag</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>candidate_tag</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -25476,16 +25569,16 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Deferred Count</t>
+          <t>Candidate Tag</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>deferred_count</t>
+          <t>candidate_tag</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -25504,16 +25597,16 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Deferral Reason</t>
+          <t>Deferred Count</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>deferral_reason</t>
+          <t>deferred_count</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -25532,16 +25625,16 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Added After Commit</t>
+          <t>Deferral Reason</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>added_after_commit</t>
+          <t>deferral_reason</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -25560,25 +25653,25 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Added After Commit</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>added_after_commit</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G194" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="195">
@@ -25588,21 +25681,21 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G195" t="n">
@@ -25616,16 +25709,16 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -25634,7 +25727,7 @@
         </is>
       </c>
       <c r="G196" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="197">
@@ -25644,16 +25737,16 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>MoSCoW</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>moscow</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -25662,7 +25755,7 @@
         </is>
       </c>
       <c r="G197" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="198">
@@ -25672,24 +25765,52 @@
         </is>
       </c>
       <c r="C198" t="n">
+        <v>14</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>MoSCoW</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>moscow</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G198" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
         <v>15</v>
       </c>
-      <c r="D198" t="inlineStr">
+      <c r="D199" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr">
+      <c r="E199" t="inlineStr">
         <is>
           <t>decision</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr">
+      <c r="F199" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="G198" t="n">
+      <c r="G199" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Priority field (P0 to P3) and pv:priority label (0.31.0)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RLE7CotBaUe74bPtiiRYNc
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N168"/>
+  <dimension ref="A1:N169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11453,6 +11453,76 @@
         <v>1</v>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>N45</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Select</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>P0 · P1 · P2 · P3</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>How urgent this is, P0 to P3: P0 = drop other work, P1 = this cycle, P2 = soon, P3 = when there is room. It is a different question from MoSCoW (whether it is in scope at all): an initiative can be a Must and still be P2. It goes to GitHub as a label and as a field of the linked GitHub Project.</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Before the push</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>New (2026-10-27)</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Asked for by Ashu (2026-10-27): P0 to P3, separate from MoSCoW, to set the Priority of the GitHub Project item and issue.</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>App -&gt; GitHub: label pv:priority/p0..p3 and the Priority field of the linked GitHub Project (single select).</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>Column on items</t>
+        </is>
+      </c>
+      <c r="N169" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11465,7 +11535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P171"/>
+  <dimension ref="A1:P172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18310,6 +18380,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>
@@ -18385,12 +18456,44 @@
     <row r="170">
       <c r="B170" t="inlineStr">
         <is>
-          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Select</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Editable</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="B171" t="inlineStr">
+        <is>
+          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" t="inlineStr">
         <is>
           <t>2026-10-23: the view columns (Prioritisation … History) on this sheet are SUPERSEDED by sheet 'Default views (ordered)' and docs/reference/default-views.csv (10 views, each with a reading order). Editing mode and the customer-safe flag on this sheet remain valid. 'In view count' is outdated.</t>
         </is>
@@ -20014,7 +20117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -20324,17 +20427,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Horizon</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>horizon</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -20352,17 +20455,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>Horizon</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>horizon</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -20380,12 +20483,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -20408,12 +20511,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Confidence-weighted Value (EUR)</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>value_weighted</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -20422,7 +20525,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -20436,12 +20539,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Confidence-weighted Value (EUR)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>value_weighted</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -20450,7 +20553,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -20464,12 +20567,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Weighted Value per Build-Week (EUR)</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>value_weighted_per_build_week</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -20478,7 +20581,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -20492,21 +20595,21 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Weighted Value per Build-Week (EUR)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>value_weighted_per_build_week</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -20520,21 +20623,21 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Crowd Rank</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>crowd_rank</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Alignment</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -20548,17 +20651,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Crowd Rank</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>crowd_rank</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Alignment</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -20576,45 +20679,40 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Planning</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Can we fit it: teams, effort by skill, estimates, dates and readiness.</t>
+          <t>Prioritisation</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -20624,11 +20722,6 @@
       </c>
       <c r="G20" t="n">
         <v>1</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="21">
@@ -20637,17 +20730,22 @@
           <t>Planning</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Can we fit it: teams, effort by skill, estimates, dates and readiness.</t>
+        </is>
+      </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -20671,16 +20769,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -20704,16 +20802,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -20723,6 +20821,11 @@
       </c>
       <c r="G23" t="n">
         <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -20732,16 +20835,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Contributing Teams</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>contributing_teams</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -20760,25 +20863,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Contributing Teams</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>contributing_teams</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -20788,16 +20891,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -20816,25 +20919,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -20844,16 +20947,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Effort by Skill</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>effort_by_skill</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -20872,16 +20975,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Estimate low (weeks)</t>
+          <t>Effort by Skill</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>estimate_low_weeks</t>
+          <t>effort_by_skill</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -20900,16 +21003,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Estimate high (weeks)</t>
+          <t>Estimate low (weeks)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>estimate_high_weeks</t>
+          <t>estimate_low_weeks</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -20928,16 +21031,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Estimate high (weeks)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>estimate_high_weeks</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -20946,7 +21049,7 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -20956,25 +21059,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Planned Start</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>planned_start</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
@@ -20984,16 +21087,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Planned Start</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>planned_start</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -21012,21 +21115,21 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Depends On (Initiative IDs)</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>depends_on</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -21040,21 +21143,21 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Depends On (Initiative IDs)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>product_manager</t>
+          <t>depends_on</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -21068,16 +21171,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>engineering_manager</t>
+          <t>product_manager</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -21096,63 +21199,53 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ready for Build</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ready_for_build</t>
+          <t>engineering_manager</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Delivery</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>How is it going: phase, health, progress, schedule, scope and engineering signals from GitHub.</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>ready_for_build</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
@@ -21161,17 +21254,22 @@
           <t>Delivery</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>How is it going: phase, health, progress, schedule, scope and engineering signals from GitHub.</t>
+        </is>
+      </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -21195,16 +21293,16 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -21228,16 +21326,16 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -21247,6 +21345,11 @@
       </c>
       <c r="G41" t="n">
         <v>1</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -21256,16 +21359,16 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -21284,16 +21387,16 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>initiative_status</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -21312,16 +21415,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -21340,16 +21443,16 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Build Status</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>description</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -21358,7 +21461,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -21368,16 +21471,16 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -21386,7 +21489,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
@@ -21396,25 +21499,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -21424,16 +21527,16 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Schedule Variance (pp)</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>schedule_variance_pp</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -21452,25 +21555,25 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Schedule Variance (pp)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>schedule_variance_pp</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -21480,16 +21583,16 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -21498,7 +21601,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -21508,25 +21611,25 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Blocked Issues (#)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>blocked_issues</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -21536,16 +21639,16 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Stale Issues (#)</t>
+          <t>Blocked Issues (#)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>stale_issues</t>
+          <t>blocked_issues</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -21564,16 +21667,16 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Scope Added (#)</t>
+          <t>Stale Issues (#)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>scope_added</t>
+          <t>stale_issues</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -21592,16 +21695,16 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Open PRs (#)</t>
+          <t>Scope Added (#)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>open_prs</t>
+          <t>scope_added</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -21620,16 +21723,16 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CI Status</t>
+          <t>Open PRs (#)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ci_status</t>
+          <t>open_prs</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -21648,16 +21751,16 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Assignees</t>
+          <t>CI Status</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>assignees</t>
+          <t>ci_status</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -21676,16 +21779,16 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Breakdown Status</t>
+          <t>Assignees</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>breakdown_status</t>
+          <t>assignees</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -21694,45 +21797,35 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Breakdown Status</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>breakdown_status</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>1</v>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -21741,17 +21834,22 @@
           <t>Go-to-market</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+        </is>
+      </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -21775,16 +21873,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -21808,16 +21906,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -21827,6 +21925,11 @@
       </c>
       <c r="G61" t="n">
         <v>1</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -21836,21 +21939,21 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Audience</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G62" t="n">
@@ -21864,25 +21967,25 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Audience</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>audience</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -21892,16 +21995,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -21910,7 +22013,7 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
@@ -21920,16 +22023,16 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Date Precision</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>date_precision</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -21948,21 +22051,21 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Target Markets</t>
+          <t>Date Precision</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>target_scope</t>
+          <t>date_precision</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G66" t="n">
@@ -21976,16 +22079,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Live Markets</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>live_scope</t>
+          <t>target_scope</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -22004,21 +22107,21 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Target Segments (customer-safe)</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>target_segments</t>
+          <t>live_scope</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -22032,21 +22135,21 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Target Customers (#)</t>
+          <t>Target Segments (customer-safe)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>target_customers</t>
+          <t>target_segments</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G69" t="n">
@@ -22060,16 +22163,16 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Customers Live (#)</t>
+          <t>Target Customers (#)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>customers_live</t>
+          <t>target_customers</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -22078,7 +22181,7 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -22088,16 +22191,16 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Roll-out %</t>
+          <t>Customers Live (#)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>rollout_pct</t>
+          <t>customers_live</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -22116,16 +22219,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Roll-out %</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>rollout_pct</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -22144,25 +22247,25 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Value Proposition (customer-safe)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>value_proposition</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G73" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74">
@@ -22172,16 +22275,16 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Value Proposition (customer-safe)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>value_proposition</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -22200,21 +22303,21 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>GTM / Enablement Notes</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>gtm_enablement_notes</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G75" t="n">
@@ -22228,21 +22331,21 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Screenshots</t>
+          <t>GTM / Enablement Notes</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>screenshots</t>
+          <t>gtm_enablement_notes</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G76" t="n">
@@ -22252,25 +22355,20 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Outcomes</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Screenshots</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>screenshots</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -22280,11 +22378,6 @@
       </c>
       <c r="G77" t="n">
         <v>1</v>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="78">
@@ -22293,17 +22386,22 @@
           <t>Outcomes</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+        </is>
+      </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -22327,16 +22425,16 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -22360,16 +22458,16 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -22379,6 +22477,11 @@
       </c>
       <c r="G80" t="n">
         <v>1</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -22388,25 +22491,25 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Outcome Status</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>outcome_status</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G81" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -22416,16 +22519,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Outcome Review Date</t>
+          <t>Outcome Status</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>outcome_review_date</t>
+          <t>outcome_status</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -22444,25 +22547,25 @@
         </is>
       </c>
       <c r="C83" t="n">
+        <v>6</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Outcome Review Date</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>outcome_review_date</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Outcomes</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
         <v>7</v>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Primary KR (Metric Name)</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>kr_metric</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="G83" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -22472,16 +22575,16 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Primary KR Unit</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>kr_unit</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -22500,16 +22603,16 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Primary KR Start Value</t>
+          <t>Primary KR Unit</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>kr_start</t>
+          <t>kr_unit</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -22528,16 +22631,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR Start Value</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_start</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -22556,25 +22659,25 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Realized KR Value</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>realized_kr_value</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G87" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -22584,16 +22687,16 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>% Realized KR Value</t>
+          <t>Realized KR Value</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>kr_realized_pct</t>
+          <t>realized_kr_value</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -22612,21 +22715,21 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>% Realized KR Value</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>kr_realized_pct</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G89" t="n">
@@ -22640,25 +22743,25 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G90" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91">
@@ -22668,25 +22771,25 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Realized EUR per year</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>realized_per_year</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G91" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -22696,16 +22799,16 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Value vs Prediction (%)</t>
+          <t>Realized EUR per year</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>value_variance_pct</t>
+          <t>realized_per_year</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -22724,16 +22827,16 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Outcome Verdict</t>
+          <t>Value vs Prediction (%)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>outcome_verdict</t>
+          <t>value_variance_pct</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -22752,16 +22855,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Time to First Use (days)</t>
+          <t>Outcome Verdict</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>time_to_first_use_days</t>
+          <t>outcome_verdict</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -22780,16 +22883,16 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Retention (%)</t>
+          <t>Time to First Use (days)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>retention_pct</t>
+          <t>time_to_first_use_days</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -22808,16 +22911,16 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Retention (%)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>retention_pct</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -22832,39 +22935,29 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Leadership</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G97" t="n">
-        <v>1</v>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="98">
@@ -22873,17 +22966,22 @@
           <t>Leadership</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+        </is>
+      </c>
       <c r="C98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -22907,16 +23005,16 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -22940,16 +23038,16 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -22959,6 +23057,11 @@
       </c>
       <c r="G100" t="n">
         <v>1</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -22968,16 +23071,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Initiative Group</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -22996,16 +23099,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Roadmap Category</t>
+          <t>Initiative Group</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>roadmap_category</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -23024,16 +23127,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Roadmap Category</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>roadmap_category</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -23052,16 +23155,16 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -23080,25 +23183,25 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G105" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -23108,25 +23211,25 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G106" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="107">
@@ -23136,16 +23239,16 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -23164,25 +23267,25 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -23192,16 +23295,16 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -23220,21 +23323,21 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G110" t="n">
@@ -23248,25 +23351,25 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Current Gate</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>current_gate</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Gates</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G111" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -23276,25 +23379,25 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Current Gate</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>current_gate</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Gates</t>
         </is>
       </c>
       <c r="G112" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="113">
@@ -23304,25 +23407,25 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>sponsor</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114">
@@ -23332,21 +23435,21 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Next Review Date</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>next_review_date</t>
+          <t>sponsor</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G114" t="n">
@@ -23360,21 +23463,21 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Next Review Date</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>next_review_date</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G115" t="n">
@@ -23384,25 +23487,20 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Discovery</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -23412,11 +23510,6 @@
       </c>
       <c r="G116" t="n">
         <v>1</v>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="117">
@@ -23425,17 +23518,22 @@
           <t>Discovery</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+        </is>
+      </c>
       <c r="C117" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -23459,16 +23557,16 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -23492,16 +23590,16 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -23511,6 +23609,11 @@
       </c>
       <c r="G119" t="n">
         <v>1</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -23520,16 +23623,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Change Type</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>change_type</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -23548,16 +23651,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
+          <t>Change Type</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>hypothesis</t>
+          <t>change_type</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -23576,21 +23679,21 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Request Origin</t>
+          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>request_origin</t>
+          <t>hypothesis</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G122" t="n">
@@ -23604,16 +23707,16 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Customers Requesting (#)</t>
+          <t>Request Origin</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>customers_requesting</t>
+          <t>request_origin</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -23632,21 +23735,21 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Customers Requesting (#)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>customers_requesting</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -23660,21 +23763,21 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Cost of Not Doing (strategic risk)</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>cost_of_not_doing</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G125" t="n">
@@ -23688,16 +23791,16 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Related / Overlaps With (Initiative IDs)</t>
+          <t>Cost of Not Doing (strategic risk)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>related_to</t>
+          <t>cost_of_not_doing</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -23716,16 +23819,16 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Dependencies / Blockers</t>
+          <t>Related / Overlaps With (Initiative IDs)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>dependencies_blockers</t>
+          <t>related_to</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -23744,16 +23847,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Dependencies / Blockers</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>dependencies_blockers</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -23772,16 +23875,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Value Type</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>value_basis</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -23800,16 +23903,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Time to First Revenue (months)</t>
+          <t>Value Basis</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>time_to_first_revenue_months</t>
+          <t>value_basis</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -23828,16 +23931,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Primary KR (Metric Name)</t>
+          <t>Time to First Revenue (months)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>kr_metric</t>
+          <t>time_to_first_revenue_months</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -23856,16 +23959,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -23884,21 +23987,21 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Artifacts (links)</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>artifacts</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G133" t="n">
@@ -23912,25 +24015,25 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Artifacts (links)</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>artifacts</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G134" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -23940,16 +24043,16 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Spec Status</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>spec_status</t>
+          <t>documents</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -23968,25 +24071,25 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Spec Status</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>product_manager</t>
+          <t>spec_status</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G136" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="137">
@@ -23996,16 +24099,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>designer</t>
+          <t>product_manager</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -24024,16 +24127,16 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>designer</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -24052,16 +24155,16 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Business Manager</t>
+          <t>Analyst</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>business_manager</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -24080,21 +24183,21 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>AI Draft (needs review)</t>
+          <t>Business Manager</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>ai_draft</t>
+          <t>business_manager</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G140" t="n">
@@ -24104,39 +24207,29 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Timeline</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+          <t>Discovery</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>AI Draft (needs review)</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>ai_draft</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G141" t="n">
         <v>1</v>
-      </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="142">
@@ -24145,17 +24238,22 @@
           <t>Timeline</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+        </is>
+      </c>
       <c r="C142" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -24179,16 +24277,16 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -24212,16 +24310,16 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -24231,6 +24329,11 @@
       </c>
       <c r="G144" t="n">
         <v>1</v>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="145">
@@ -24240,25 +24343,25 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Days in Current Phase</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>days_in_phase</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G145" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
@@ -24268,25 +24371,25 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Days in Current Phase</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>days_in_phase</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
@@ -24296,16 +24399,16 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Start Discovery</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>start_discovery</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -24324,16 +24427,16 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Start Definition</t>
+          <t>Start Discovery</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>start_definition</t>
+          <t>start_discovery</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -24352,16 +24455,16 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Start Building</t>
+          <t>Start Definition</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>start_building</t>
+          <t>start_definition</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -24380,16 +24483,16 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Start Beta-Test</t>
+          <t>Start Building</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>start_beta</t>
+          <t>start_building</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -24408,16 +24511,16 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Start Experiment</t>
+          <t>Start Beta-Test</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>start_experiment</t>
+          <t>start_beta</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -24436,16 +24539,16 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Start Roll-Out</t>
+          <t>Start Experiment</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>start_rollout</t>
+          <t>start_experiment</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -24464,16 +24567,16 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>G2M Date (actual)</t>
+          <t>Start Roll-Out</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>g2m_date_actual</t>
+          <t>start_rollout</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -24492,25 +24595,25 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Discovery Time (days)</t>
+          <t>G2M Date (actual)</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>time_discovery_days</t>
+          <t>g2m_date_actual</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G154" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
@@ -24520,16 +24623,16 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Definition Time (days)</t>
+          <t>Discovery Time (days)</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>time_definition_days</t>
+          <t>time_discovery_days</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -24548,16 +24651,16 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Building Time (days)</t>
+          <t>Definition Time (days)</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>time_building_days</t>
+          <t>time_definition_days</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -24576,16 +24679,16 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Beta-Test Time (days)</t>
+          <t>Building Time (days)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>time_beta_days</t>
+          <t>time_building_days</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -24604,16 +24707,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Experiment Time (days)</t>
+          <t>Beta-Test Time (days)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>time_experiment_days</t>
+          <t>time_beta_days</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -24632,16 +24735,16 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Roll-Out Time (days)</t>
+          <t>Experiment Time (days)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>time_rollout_days</t>
+          <t>time_experiment_days</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -24660,16 +24763,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Time to Market (days)</t>
+          <t>Roll-Out Time (days)</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>time_to_market_days</t>
+          <t>time_rollout_days</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -24688,16 +24791,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Actual Build (weeks)</t>
+          <t>Time to Market (days)</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>actual_build_weeks</t>
+          <t>time_to_market_days</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -24716,16 +24819,16 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Build vs Estimate High (%)</t>
+          <t>Actual Build (weeks)</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>build_vs_estimate_high_pct</t>
+          <t>actual_build_weeks</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -24744,16 +24847,16 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Blocked Days</t>
+          <t>Build vs Estimate High (%)</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>blocked_days</t>
+          <t>build_vs_estimate_high_pct</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -24768,39 +24871,29 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>History</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Blocked Days</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>blocked_days</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G164" t="n">
-        <v>1</v>
-      </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="165">
@@ -24809,17 +24902,22 @@
           <t>History</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+        </is>
+      </c>
       <c r="C165" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -24843,16 +24941,16 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -24876,16 +24974,16 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>initiative_status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -24895,6 +24993,11 @@
       </c>
       <c r="G167" t="n">
         <v>1</v>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="168">
@@ -24904,16 +25007,16 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Build Status</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -24922,7 +25025,7 @@
         </is>
       </c>
       <c r="G168" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169">
@@ -24932,16 +25035,16 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -24950,7 +25053,7 @@
         </is>
       </c>
       <c r="G169" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="170">
@@ -24960,16 +25063,16 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -24988,21 +25091,21 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G171" t="n">
@@ -25016,16 +25119,16 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Decided By</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>decided_by</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -25044,16 +25147,16 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Decision Date</t>
+          <t>Decided By</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>decision_date</t>
+          <t>decided_by</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -25072,21 +25175,21 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Status Changed At</t>
+          <t>Decision Date</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>status_changed_at</t>
+          <t>decision_date</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G174" t="n">
@@ -25100,16 +25203,16 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Phase Changed At</t>
+          <t>Status Changed At</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>phase_changed_at</t>
+          <t>status_changed_at</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -25128,21 +25231,21 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>Phase Changed At</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>last_edited_at</t>
+          <t>phase_changed_at</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G176" t="n">
@@ -25156,21 +25259,21 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Last Edited By</t>
+          <t>Last Updated</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>last_edited_by</t>
+          <t>last_edited_at</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G177" t="n">
@@ -25184,16 +25287,16 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Created At</t>
+          <t>Last Edited By</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>last_edited_by</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -25212,16 +25315,16 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Created By</t>
+          <t>Created At</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -25240,16 +25343,16 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Created Via</t>
+          <t>Created By</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>created_via</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -25268,16 +25371,16 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Last Reviewed</t>
+          <t>Created Via</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>last_reviewed_at</t>
+          <t>created_via</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -25296,16 +25399,16 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Review Overdue</t>
+          <t>Last Reviewed</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>review_overdue</t>
+          <t>last_reviewed_at</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -25314,7 +25417,7 @@
         </is>
       </c>
       <c r="G182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -25324,16 +25427,16 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Item Age (days)</t>
+          <t>Review Overdue</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>item_age_days</t>
+          <t>review_overdue</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -25352,16 +25455,16 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Archived</t>
+          <t>Item Age (days)</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>item_age_days</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -25370,45 +25473,35 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Cycle review</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>archived</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G185" t="n">
         <v>1</v>
-      </c>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="186">
@@ -25417,17 +25510,22 @@
           <t>Cycle review</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+        </is>
+      </c>
       <c r="C186" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -25451,16 +25549,16 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -25484,16 +25582,16 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -25503,6 +25601,11 @@
       </c>
       <c r="G188" t="n">
         <v>1</v>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="189">
@@ -25512,25 +25615,25 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G189" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190">
@@ -25540,16 +25643,16 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -25568,16 +25671,16 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Candidate Tag</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>candidate_tag</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -25596,16 +25699,16 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Deferred Count</t>
+          <t>Candidate Tag</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>deferred_count</t>
+          <t>candidate_tag</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -25624,16 +25727,16 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Deferral Reason</t>
+          <t>Deferred Count</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>deferral_reason</t>
+          <t>deferred_count</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -25652,16 +25755,16 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Added After Commit</t>
+          <t>Deferral Reason</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>added_after_commit</t>
+          <t>deferral_reason</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -25680,25 +25783,25 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Added After Commit</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>added_after_commit</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G195" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="196">
@@ -25708,21 +25811,21 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G196" t="n">
@@ -25736,16 +25839,16 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -25754,7 +25857,7 @@
         </is>
       </c>
       <c r="G197" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198">
@@ -25764,16 +25867,16 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>MoSCoW</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>moscow</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -25782,7 +25885,7 @@
         </is>
       </c>
       <c r="G198" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="199">
@@ -25792,24 +25895,80 @@
         </is>
       </c>
       <c r="C199" t="n">
+        <v>14</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>MoSCoW</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>moscow</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G199" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
         <v>15</v>
       </c>
-      <c r="D199" t="inlineStr">
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G200" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>16</v>
+      </c>
+      <c r="D201" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr">
+      <c r="E201" t="inlineStr">
         <is>
           <t>decision</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="F201" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="G199" t="n">
+      <c r="G201" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Last Synced and Synced With columns and a panel line (0.33.0)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RLE7CotBaUe74bPtiiRYNc
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N168"/>
+  <dimension ref="A1:N170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11453,6 +11453,136 @@
         <v>1</v>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>N46</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Delivery (GitHub)</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Last Synced</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>last_synced</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>When this initiative was last in step with its tracker: the latest of the last confirmed send and the last time GitHub's changes were applied. Empty when it is not on a tracker.</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>After the first send or check</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>New (2026-10-27)</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Asked for by Ashu (2026-10-27): see when a line was last synced and with what.</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Not synced: shown from the GitHub link, read-only.</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>Derived in the app from the GitHub link (not stored)</t>
+        </is>
+      </c>
+      <c r="N169" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>N47</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Delivery (GitHub)</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Synced With</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>synced_with</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Where this initiative syncs to, for example GitHub, the repository, and the Project board it is on. Says when the last send failed or when it only follows an issue read-only.</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>After the first send or check</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>New (2026-10-27)</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Asked for by Ashu (2026-10-27): the platform and place, next to the time.</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Not synced: shown from the GitHub link, read-only.</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>Derived in the app from the GitHub link (not stored)</t>
+        </is>
+      </c>
+      <c r="N170" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11465,7 +11595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P171"/>
+  <dimension ref="A1:P173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18385,12 +18515,76 @@
     <row r="170">
       <c r="B170" t="inlineStr">
         <is>
-          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+          <t>Last Synced</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>last_synced</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Delivery (GitHub)</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Computed (read-only)</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="B171" t="inlineStr">
+        <is>
+          <t>Synced With</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>synced_with</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Delivery (GitHub)</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Computed (read-only)</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" t="inlineStr">
         <is>
           <t>2026-10-23: the view columns (Prioritisation … History) on this sheet are SUPERSEDED by sheet 'Default views (ordered)' and docs/reference/default-views.csv (10 views, each with a reading order). Editing mode and the customer-safe flag on this sheet remain valid. 'In view count' is outdated.</t>
         </is>
@@ -20014,7 +20208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21372,17 +21566,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Last Synced</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>last_synced</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G46" t="n">
@@ -21400,12 +21594,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Synced With</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>synced_with</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -21414,7 +21608,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -21428,21 +21622,21 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Schedule Variance (pp)</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>schedule_variance_pp</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -21456,21 +21650,21 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -21484,21 +21678,21 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>Schedule Variance (pp)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>schedule_variance_pp</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -21512,21 +21706,21 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Blocked Issues (#)</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>blocked_issues</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -21540,21 +21734,21 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Stale Issues (#)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>stale_issues</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -21568,12 +21762,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Scope Added (#)</t>
+          <t>Blocked Issues (#)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>scope_added</t>
+          <t>blocked_issues</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -21596,12 +21790,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Open PRs (#)</t>
+          <t>Stale Issues (#)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>open_prs</t>
+          <t>stale_issues</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -21624,12 +21818,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CI Status</t>
+          <t>Scope Added (#)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ci_status</t>
+          <t>scope_added</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -21652,12 +21846,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Assignees</t>
+          <t>Open PRs (#)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>assignees</t>
+          <t>open_prs</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -21680,12 +21874,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Breakdown Status</t>
+          <t>CI Status</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>breakdown_status</t>
+          <t>ci_status</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -21694,78 +21888,63 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Assignees</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>assignees</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>1</v>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Breakdown Status</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>breakdown_status</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>1</v>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="60">
@@ -21774,17 +21953,22 @@
           <t>Go-to-market</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+        </is>
+      </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -21808,16 +21992,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -21827,6 +22011,11 @@
       </c>
       <c r="G61" t="n">
         <v>1</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -21836,25 +22025,30 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Audience</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G62" t="n">
         <v>1</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -21864,25 +22058,25 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -21892,21 +22086,21 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Audience</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>audience</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G64" t="n">
@@ -21920,16 +22114,16 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Date Precision</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>date_precision</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -21938,7 +22132,7 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
@@ -21948,21 +22142,21 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Target Markets</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>target_scope</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G66" t="n">
@@ -21976,21 +22170,21 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Live Markets</t>
+          <t>Date Precision</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>live_scope</t>
+          <t>date_precision</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G67" t="n">
@@ -22004,21 +22198,21 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Target Segments (customer-safe)</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>target_segments</t>
+          <t>target_scope</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -22032,16 +22226,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Target Customers (#)</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>target_customers</t>
+          <t>live_scope</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -22060,25 +22254,25 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Customers Live (#)</t>
+          <t>Target Segments (customer-safe)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>customers_live</t>
+          <t>target_segments</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G70" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -22088,16 +22282,16 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Roll-out %</t>
+          <t>Target Customers (#)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>rollout_pct</t>
+          <t>target_customers</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -22106,7 +22300,7 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -22116,16 +22310,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Customers Live (#)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>customers_live</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -22144,25 +22338,25 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Value Proposition (customer-safe)</t>
+          <t>Roll-out %</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>value_proposition</t>
+          <t>rollout_pct</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G73" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74">
@@ -22172,25 +22366,25 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G74" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="75">
@@ -22200,21 +22394,21 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>GTM / Enablement Notes</t>
+          <t>Value Proposition (customer-safe)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>gtm_enablement_notes</t>
+          <t>value_proposition</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G75" t="n">
@@ -22228,16 +22422,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Screenshots</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>screenshots</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -22252,58 +22446,48 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Outcomes</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>GTM / Enablement Notes</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>gtm_enablement_notes</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G77" t="n">
         <v>1</v>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Screenshots</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>screenshots</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -22313,11 +22497,6 @@
       </c>
       <c r="G78" t="n">
         <v>1</v>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="79">
@@ -22326,17 +22505,22 @@
           <t>Outcomes</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+        </is>
+      </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -22360,16 +22544,16 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -22379,6 +22563,11 @@
       </c>
       <c r="G80" t="n">
         <v>1</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -22388,25 +22577,30 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Outcome Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>outcome_status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G81" t="n">
-        <v>7</v>
+        <v>1</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -22416,25 +22610,25 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Outcome Review Date</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>outcome_review_date</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G82" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -22444,25 +22638,25 @@
         </is>
       </c>
       <c r="C83" t="n">
+        <v>5</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Outcome Status</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>outcome_status</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Outcomes</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
         <v>7</v>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Primary KR (Metric Name)</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>kr_metric</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="G83" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -22472,25 +22666,25 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Primary KR Unit</t>
+          <t>Outcome Review Date</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>kr_unit</t>
+          <t>outcome_review_date</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G84" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="85">
@@ -22500,16 +22694,16 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Primary KR Start Value</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>kr_start</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -22528,16 +22722,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR Unit</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_unit</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -22556,25 +22750,25 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Realized KR Value</t>
+          <t>Primary KR Start Value</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>realized_kr_value</t>
+          <t>kr_start</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G87" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -22584,25 +22778,25 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>% Realized KR Value</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>kr_realized_pct</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G88" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -22612,21 +22806,21 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Realized KR Value</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>realized_kr_value</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G89" t="n">
@@ -22640,25 +22834,25 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>% Realized KR Value</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>kr_realized_pct</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G90" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91">
@@ -22668,21 +22862,21 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Realized EUR per year</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>realized_per_year</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G91" t="n">
@@ -22696,25 +22890,25 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Value vs Prediction (%)</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>value_variance_pct</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G92" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -22724,16 +22918,16 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Outcome Verdict</t>
+          <t>Realized EUR per year</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>outcome_verdict</t>
+          <t>realized_per_year</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -22752,16 +22946,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Time to First Use (days)</t>
+          <t>Value vs Prediction (%)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>time_to_first_use_days</t>
+          <t>value_variance_pct</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -22780,16 +22974,16 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Retention (%)</t>
+          <t>Outcome Verdict</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>retention_pct</t>
+          <t>outcome_verdict</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -22808,16 +23002,16 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Time to First Use (days)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>time_to_first_use_days</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -22832,72 +23026,57 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Leadership</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Retention (%)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>retention_pct</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G97" t="n">
-        <v>1</v>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Leadership</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G98" t="n">
-        <v>1</v>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="99">
@@ -22906,17 +23085,22 @@
           <t>Leadership</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+        </is>
+      </c>
       <c r="C99" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -22940,16 +23124,16 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -22959,6 +23143,11 @@
       </c>
       <c r="G100" t="n">
         <v>1</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -22968,16 +23157,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Initiative Group</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -22987,6 +23176,11 @@
       </c>
       <c r="G101" t="n">
         <v>1</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -22996,16 +23190,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Roadmap Category</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>roadmap_category</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -23024,16 +23218,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Group</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -23052,16 +23246,16 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Roadmap Category</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>roadmap_category</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -23080,25 +23274,25 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G105" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -23108,25 +23302,25 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -23136,25 +23330,25 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108">
@@ -23164,25 +23358,25 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -23192,25 +23386,25 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110">
@@ -23220,21 +23414,21 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G110" t="n">
@@ -23248,25 +23442,25 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Current Gate</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>current_gate</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Gates</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G111" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -23276,25 +23470,25 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G112" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -23304,25 +23498,25 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Current Gate</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>sponsor</t>
+          <t>current_gate</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Gates</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114">
@@ -23332,25 +23526,25 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Next Review Date</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>next_review_date</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="115">
@@ -23360,21 +23554,21 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>sponsor</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G115" t="n">
@@ -23384,58 +23578,48 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Discovery</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Next Review Date</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>next_review_date</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G116" t="n">
         <v>1</v>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Discovery</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -23445,11 +23629,6 @@
       </c>
       <c r="G117" t="n">
         <v>1</v>
-      </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="118">
@@ -23458,17 +23637,22 @@
           <t>Discovery</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+        </is>
+      </c>
       <c r="C118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -23492,16 +23676,16 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -23511,6 +23695,11 @@
       </c>
       <c r="G119" t="n">
         <v>1</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -23520,16 +23709,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Change Type</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>change_type</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -23539,6 +23728,11 @@
       </c>
       <c r="G120" t="n">
         <v>1</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -23548,16 +23742,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>hypothesis</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -23576,21 +23770,21 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Request Origin</t>
+          <t>Change Type</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>request_origin</t>
+          <t>change_type</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G122" t="n">
@@ -23604,21 +23798,21 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Customers Requesting (#)</t>
+          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>customers_requesting</t>
+          <t>hypothesis</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G123" t="n">
@@ -23632,21 +23826,21 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Request Origin</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>request_origin</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -23660,21 +23854,21 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Cost of Not Doing (strategic risk)</t>
+          <t>Customers Requesting (#)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>cost_of_not_doing</t>
+          <t>customers_requesting</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G125" t="n">
@@ -23688,21 +23882,21 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Related / Overlaps With (Initiative IDs)</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>related_to</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G126" t="n">
@@ -23716,16 +23910,16 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Dependencies / Blockers</t>
+          <t>Cost of Not Doing (strategic risk)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>dependencies_blockers</t>
+          <t>cost_of_not_doing</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -23744,16 +23938,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Related / Overlaps With (Initiative IDs)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>related_to</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -23772,16 +23966,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Dependencies / Blockers</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>value_basis</t>
+          <t>dependencies_blockers</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -23800,16 +23994,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Time to First Revenue (months)</t>
+          <t>Value Type</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>time_to_first_revenue_months</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -23828,16 +24022,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Primary KR (Metric Name)</t>
+          <t>Value Basis</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>kr_metric</t>
+          <t>value_basis</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -23856,16 +24050,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Time to First Revenue (months)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>time_to_first_revenue_months</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -23884,21 +24078,21 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Artifacts (links)</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>artifacts</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G133" t="n">
@@ -23912,25 +24106,25 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G134" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -23940,25 +24134,25 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Spec Status</t>
+          <t>Artifacts (links)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>spec_status</t>
+          <t>artifacts</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G135" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136">
@@ -23968,25 +24162,25 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>product_manager</t>
+          <t>documents</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G136" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="137">
@@ -23996,25 +24190,25 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Spec Status</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>designer</t>
+          <t>spec_status</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G137" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="138">
@@ -24024,16 +24218,16 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>product_manager</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -24052,16 +24246,16 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Business Manager</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>business_manager</t>
+          <t>designer</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -24080,21 +24274,21 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>AI Draft (needs review)</t>
+          <t>Analyst</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>ai_draft</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G140" t="n">
@@ -24104,72 +24298,57 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Timeline</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+          <t>Discovery</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Business Manager</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>business_manager</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G141" t="n">
         <v>1</v>
-      </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Timeline</t>
+          <t>Discovery</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>AI Draft (needs review)</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>ai_draft</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G142" t="n">
         <v>1</v>
-      </c>
-      <c r="H142" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="143">
@@ -24178,17 +24357,22 @@
           <t>Timeline</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+        </is>
+      </c>
       <c r="C143" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -24212,16 +24396,16 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -24231,6 +24415,11 @@
       </c>
       <c r="G144" t="n">
         <v>1</v>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="145">
@@ -24240,25 +24429,30 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Days in Current Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>days_in_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G145" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="146">
@@ -24268,21 +24462,21 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G146" t="n">
@@ -24296,25 +24490,25 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Start Discovery</t>
+          <t>Days in Current Phase</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>start_discovery</t>
+          <t>days_in_phase</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148">
@@ -24324,16 +24518,16 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Start Definition</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>start_definition</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -24352,16 +24546,16 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Start Building</t>
+          <t>Start Discovery</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>start_building</t>
+          <t>start_discovery</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -24380,16 +24574,16 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Start Beta-Test</t>
+          <t>Start Definition</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>start_beta</t>
+          <t>start_definition</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -24408,16 +24602,16 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Start Experiment</t>
+          <t>Start Building</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>start_experiment</t>
+          <t>start_building</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -24436,16 +24630,16 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Start Roll-Out</t>
+          <t>Start Beta-Test</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>start_rollout</t>
+          <t>start_beta</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -24464,16 +24658,16 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>G2M Date (actual)</t>
+          <t>Start Experiment</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>g2m_date_actual</t>
+          <t>start_experiment</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -24492,25 +24686,25 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Discovery Time (days)</t>
+          <t>Start Roll-Out</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>time_discovery_days</t>
+          <t>start_rollout</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G154" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
@@ -24520,25 +24714,25 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Definition Time (days)</t>
+          <t>G2M Date (actual)</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>time_definition_days</t>
+          <t>g2m_date_actual</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G155" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -24548,16 +24742,16 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Building Time (days)</t>
+          <t>Discovery Time (days)</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>time_building_days</t>
+          <t>time_discovery_days</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -24576,16 +24770,16 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Beta-Test Time (days)</t>
+          <t>Definition Time (days)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>time_beta_days</t>
+          <t>time_definition_days</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -24604,16 +24798,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Experiment Time (days)</t>
+          <t>Building Time (days)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>time_experiment_days</t>
+          <t>time_building_days</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -24632,16 +24826,16 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Roll-Out Time (days)</t>
+          <t>Beta-Test Time (days)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>time_rollout_days</t>
+          <t>time_beta_days</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -24660,16 +24854,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Time to Market (days)</t>
+          <t>Experiment Time (days)</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>time_to_market_days</t>
+          <t>time_experiment_days</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -24688,16 +24882,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Actual Build (weeks)</t>
+          <t>Roll-Out Time (days)</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>actual_build_weeks</t>
+          <t>time_rollout_days</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -24716,16 +24910,16 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Build vs Estimate High (%)</t>
+          <t>Time to Market (days)</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>build_vs_estimate_high_pct</t>
+          <t>time_to_market_days</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -24744,16 +24938,16 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Blocked Days</t>
+          <t>Actual Build (weeks)</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>blocked_days</t>
+          <t>actual_build_weeks</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -24768,72 +24962,57 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>History</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Build vs Estimate High (%)</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>build_vs_estimate_high_pct</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G164" t="n">
-        <v>1</v>
-      </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Blocked Days</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>blocked_days</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G165" t="n">
-        <v>1</v>
-      </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="166">
@@ -24842,17 +25021,22 @@
           <t>History</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+        </is>
+      </c>
       <c r="C166" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -24876,16 +25060,16 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>initiative_status</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -24895,6 +25079,11 @@
       </c>
       <c r="G167" t="n">
         <v>1</v>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="168">
@@ -24904,16 +25093,16 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Build Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -24922,7 +25111,12 @@
         </is>
       </c>
       <c r="G168" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="169">
@@ -24932,16 +25126,16 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -24960,16 +25154,16 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -24978,7 +25172,7 @@
         </is>
       </c>
       <c r="G170" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171">
@@ -24988,21 +25182,21 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G171" t="n">
@@ -25016,21 +25210,21 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Decided By</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>decided_by</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G172" t="n">
@@ -25044,16 +25238,16 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Decision Date</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>decision_date</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -25072,21 +25266,21 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Status Changed At</t>
+          <t>Decided By</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>status_changed_at</t>
+          <t>decided_by</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G174" t="n">
@@ -25100,21 +25294,21 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Phase Changed At</t>
+          <t>Decision Date</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>phase_changed_at</t>
+          <t>decision_date</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G175" t="n">
@@ -25128,21 +25322,21 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>Status Changed At</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>last_edited_at</t>
+          <t>status_changed_at</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G176" t="n">
@@ -25156,16 +25350,16 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Last Edited By</t>
+          <t>Phase Changed At</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>last_edited_by</t>
+          <t>phase_changed_at</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -25184,21 +25378,21 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Created At</t>
+          <t>Last Updated</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>last_edited_at</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G178" t="n">
@@ -25212,16 +25406,16 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Created By</t>
+          <t>Last Edited By</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>last_edited_by</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -25240,16 +25434,16 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Created Via</t>
+          <t>Created At</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>created_via</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -25268,16 +25462,16 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Last Reviewed</t>
+          <t>Created By</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>last_reviewed_at</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -25296,16 +25490,16 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Review Overdue</t>
+          <t>Created Via</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>review_overdue</t>
+          <t>created_via</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -25314,7 +25508,7 @@
         </is>
       </c>
       <c r="G182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -25324,16 +25518,16 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Item Age (days)</t>
+          <t>Last Reviewed</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>item_age_days</t>
+          <t>last_reviewed_at</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -25342,7 +25536,7 @@
         </is>
       </c>
       <c r="G183" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184">
@@ -25352,16 +25546,16 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Archived</t>
+          <t>Review Overdue</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>review_overdue</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -25370,78 +25564,63 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Cycle review</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Item Age (days)</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_age_days</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G185" t="n">
-        <v>1</v>
-      </c>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Cycle review</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>archived</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G186" t="n">
         <v>1</v>
-      </c>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="187">
@@ -25450,17 +25629,22 @@
           <t>Cycle review</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+        </is>
+      </c>
       <c r="C187" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -25484,16 +25668,16 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -25503,6 +25687,11 @@
       </c>
       <c r="G188" t="n">
         <v>1</v>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="189">
@@ -25512,25 +25701,30 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G189" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="190">
@@ -25540,25 +25734,25 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G190" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="191">
@@ -25568,16 +25762,16 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Candidate Tag</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>candidate_tag</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -25596,16 +25790,16 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Deferred Count</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>deferred_count</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -25624,16 +25818,16 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Deferral Reason</t>
+          <t>Candidate Tag</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>deferral_reason</t>
+          <t>candidate_tag</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -25652,16 +25846,16 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Added After Commit</t>
+          <t>Deferred Count</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>added_after_commit</t>
+          <t>deferred_count</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -25680,25 +25874,25 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Deferral Reason</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>deferral_reason</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G195" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="196">
@@ -25708,25 +25902,25 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Added After Commit</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>added_after_commit</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G196" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="197">
@@ -25736,25 +25930,25 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G197" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198">
@@ -25764,16 +25958,16 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>MoSCoW</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>moscow</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -25792,24 +25986,80 @@
         </is>
       </c>
       <c r="C199" t="n">
+        <v>13</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Fit by Team</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>fit_by_team</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G199" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>14</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>MoSCoW</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>moscow</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G200" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
         <v>15</v>
       </c>
-      <c r="D199" t="inlineStr">
+      <c r="D201" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr">
+      <c r="E201" t="inlineStr">
         <is>
           <t>decision</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="F201" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="G199" t="n">
+      <c r="G201" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP: Delivery Status (board status read back)
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>Project Status (GitHub)</t>
+          <t>Delivery Status</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
@@ -6921,19 +6921,15 @@
           <t>Computed</t>
         </is>
       </c>
-      <c r="F100" s="9" t="inlineStr">
-        <is>
-          <t>As defined in the linked GitHub Project (e.g. Todo · In Progress · Done)</t>
-        </is>
-      </c>
+      <c r="F100" s="9" t="n"/>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>Value of the Status field of the item in the linked GitHub Project.</t>
+          <t>Where the initiative stands on the linked GitHub Project board, in the board's own words (for example Backlog, Ready, In progress, On staging, Done). Read from the board, never written by Product Velocity, and separate from Build Status (the issue's open or closed state) and from Initiative Status (set by people).</t>
         </is>
       </c>
       <c r="H100" s="9" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>After the initiative is on the board</t>
         </is>
       </c>
       <c r="I100" s="9" t="inlineStr">
@@ -6943,17 +6939,17 @@
       </c>
       <c r="J100" s="14" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Renamed and brought forward (2026-10-27)</t>
         </is>
       </c>
       <c r="K100" s="9" t="inlineStr">
         <is>
-          <t>Shows what engineering sees on their board. Needs a linked org-owned GitHub Project.</t>
+          <t>Ashu (2026-10-27): the board's Status is the delivery status; PV's own status is not mapped to GitHub. Free text from the board, no mapping table.</t>
         </is>
       </c>
       <c r="L100" s="9" t="inlineStr">
         <is>
-          <t>Projects v2 -&gt; app, read-only.</t>
+          <t>Projects v2 -&gt; app, read-only (the board's Status field, in real time through the projects_v2_item event and at every check).</t>
         </is>
       </c>
       <c r="M100" s="9" t="inlineStr">
@@ -6962,7 +6958,7 @@
         </is>
       </c>
       <c r="N100" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -15688,7 +15684,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Project Status (GitHub)</t>
+          <t>Delivery Status</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -18440,6 +18436,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>
@@ -20208,7 +20205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21566,12 +21563,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Last Synced</t>
+          <t>Delivery Status</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>last_synced</t>
+          <t>gh_project_status</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -21594,12 +21591,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Synced With</t>
+          <t>Last Synced</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>synced_with</t>
+          <t>last_synced</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -21622,17 +21619,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Synced With</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>synced_with</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G48" t="n">
@@ -21650,21 +21647,21 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -21678,12 +21675,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Schedule Variance (pp)</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>schedule_variance_pp</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -21706,21 +21703,21 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Schedule Variance (pp)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>schedule_variance_pp</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -21734,12 +21731,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -21748,7 +21745,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -21762,21 +21759,21 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Blocked Issues (#)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>blocked_issues</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -21790,12 +21787,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Stale Issues (#)</t>
+          <t>Blocked Issues (#)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>stale_issues</t>
+          <t>blocked_issues</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -21818,12 +21815,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Scope Added (#)</t>
+          <t>Stale Issues (#)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>scope_added</t>
+          <t>stale_issues</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -21846,12 +21843,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Open PRs (#)</t>
+          <t>Scope Added (#)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>open_prs</t>
+          <t>scope_added</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -21874,12 +21871,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CI Status</t>
+          <t>Open PRs (#)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ci_status</t>
+          <t>open_prs</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -21902,12 +21899,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Assignees</t>
+          <t>CI Status</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>assignees</t>
+          <t>ci_status</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -21930,12 +21927,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Breakdown Status</t>
+          <t>Assignees</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>breakdown_status</t>
+          <t>assignees</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -21944,45 +21941,35 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Breakdown Status</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>breakdown_status</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>1</v>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="61">
@@ -21991,17 +21978,22 @@
           <t>Go-to-market</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+        </is>
+      </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -22025,16 +22017,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -22058,16 +22050,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -22077,6 +22069,11 @@
       </c>
       <c r="G63" t="n">
         <v>1</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -22086,21 +22083,21 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Audience</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G64" t="n">
@@ -22114,25 +22111,25 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Audience</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>audience</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -22142,16 +22139,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -22160,7 +22157,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67">
@@ -22170,16 +22167,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Date Precision</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>date_precision</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -22198,21 +22195,21 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Target Markets</t>
+          <t>Date Precision</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>target_scope</t>
+          <t>date_precision</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -22226,16 +22223,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Live Markets</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>live_scope</t>
+          <t>target_scope</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -22254,21 +22251,21 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Target Segments (customer-safe)</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>target_segments</t>
+          <t>live_scope</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G70" t="n">
@@ -22282,21 +22279,21 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Target Customers (#)</t>
+          <t>Target Segments (customer-safe)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>target_customers</t>
+          <t>target_segments</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G71" t="n">
@@ -22310,16 +22307,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Customers Live (#)</t>
+          <t>Target Customers (#)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>customers_live</t>
+          <t>target_customers</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -22328,7 +22325,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -22338,16 +22335,16 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Roll-out %</t>
+          <t>Customers Live (#)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>rollout_pct</t>
+          <t>customers_live</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -22366,16 +22363,16 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Roll-out %</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>rollout_pct</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -22394,25 +22391,25 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Value Proposition (customer-safe)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>value_proposition</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G75" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76">
@@ -22422,16 +22419,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Value Proposition (customer-safe)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>value_proposition</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -22450,21 +22447,21 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>GTM / Enablement Notes</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>gtm_enablement_notes</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G77" t="n">
@@ -22478,21 +22475,21 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Screenshots</t>
+          <t>GTM / Enablement Notes</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>screenshots</t>
+          <t>gtm_enablement_notes</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G78" t="n">
@@ -22502,25 +22499,20 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Outcomes</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Screenshots</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>screenshots</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -22530,11 +22522,6 @@
       </c>
       <c r="G79" t="n">
         <v>1</v>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="80">
@@ -22543,17 +22530,22 @@
           <t>Outcomes</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+        </is>
+      </c>
       <c r="C80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -22577,16 +22569,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -22610,16 +22602,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -22629,6 +22621,11 @@
       </c>
       <c r="G82" t="n">
         <v>1</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -22638,25 +22635,25 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Outcome Status</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>outcome_status</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G83" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -22666,16 +22663,16 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Outcome Review Date</t>
+          <t>Outcome Status</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>outcome_review_date</t>
+          <t>outcome_status</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -22694,25 +22691,25 @@
         </is>
       </c>
       <c r="C85" t="n">
+        <v>6</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Outcome Review Date</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>outcome_review_date</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Outcomes</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
         <v>7</v>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Primary KR (Metric Name)</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>kr_metric</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="G85" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -22722,16 +22719,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Primary KR Unit</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>kr_unit</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -22750,16 +22747,16 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Primary KR Start Value</t>
+          <t>Primary KR Unit</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>kr_start</t>
+          <t>kr_unit</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -22778,16 +22775,16 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR Start Value</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_start</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -22806,25 +22803,25 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Realized KR Value</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>realized_kr_value</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -22834,16 +22831,16 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>% Realized KR Value</t>
+          <t>Realized KR Value</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>kr_realized_pct</t>
+          <t>realized_kr_value</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -22862,21 +22859,21 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>% Realized KR Value</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>kr_realized_pct</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G91" t="n">
@@ -22890,25 +22887,25 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="93">
@@ -22918,25 +22915,25 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Realized EUR per year</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>realized_per_year</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G93" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -22946,16 +22943,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Value vs Prediction (%)</t>
+          <t>Realized EUR per year</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>value_variance_pct</t>
+          <t>realized_per_year</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -22974,16 +22971,16 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Outcome Verdict</t>
+          <t>Value vs Prediction (%)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>outcome_verdict</t>
+          <t>value_variance_pct</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -23002,16 +22999,16 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Time to First Use (days)</t>
+          <t>Outcome Verdict</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>time_to_first_use_days</t>
+          <t>outcome_verdict</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -23030,16 +23027,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Retention (%)</t>
+          <t>Time to First Use (days)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>retention_pct</t>
+          <t>time_to_first_use_days</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -23058,16 +23055,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Retention (%)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>retention_pct</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -23082,39 +23079,29 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Leadership</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G99" t="n">
-        <v>1</v>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="100">
@@ -23123,17 +23110,22 @@
           <t>Leadership</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+        </is>
+      </c>
       <c r="C100" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -23157,16 +23149,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -23190,16 +23182,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -23209,6 +23201,11 @@
       </c>
       <c r="G102" t="n">
         <v>1</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -23218,16 +23215,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Initiative Group</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -23246,16 +23243,16 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Roadmap Category</t>
+          <t>Initiative Group</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>roadmap_category</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -23274,16 +23271,16 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Roadmap Category</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>roadmap_category</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -23302,16 +23299,16 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -23330,25 +23327,25 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -23358,25 +23355,25 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="109">
@@ -23386,16 +23383,16 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Quarter</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -23414,25 +23411,25 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111">
@@ -23442,16 +23439,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Value (EUR, 12-month run-rate)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -23470,21 +23467,21 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G112" t="n">
@@ -23498,25 +23495,25 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Current Gate</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>current_gate</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Gates</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -23526,25 +23523,25 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Current Gate</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>current_gate</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Gates</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115">
@@ -23554,25 +23551,25 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>sponsor</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="116">
@@ -23582,21 +23579,21 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Next Review Date</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>next_review_date</t>
+          <t>sponsor</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G116" t="n">
@@ -23610,21 +23607,21 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Next Review Date</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>next_review_date</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G117" t="n">
@@ -23634,25 +23631,20 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Discovery</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -23662,11 +23654,6 @@
       </c>
       <c r="G118" t="n">
         <v>1</v>
-      </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="119">
@@ -23675,17 +23662,22 @@
           <t>Discovery</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+        </is>
+      </c>
       <c r="C119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -23709,16 +23701,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -23742,16 +23734,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -23761,6 +23753,11 @@
       </c>
       <c r="G121" t="n">
         <v>1</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -23770,16 +23767,16 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Change Type</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>change_type</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -23798,16 +23795,16 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
+          <t>Change Type</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>hypothesis</t>
+          <t>change_type</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -23826,21 +23823,21 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Request Origin</t>
+          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>request_origin</t>
+          <t>hypothesis</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -23854,16 +23851,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Customers Requesting (#)</t>
+          <t>Request Origin</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>customers_requesting</t>
+          <t>request_origin</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -23882,21 +23879,21 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Customers Requesting (#)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>customers_requesting</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G126" t="n">
@@ -23910,21 +23907,21 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Cost of Not Doing (strategic risk)</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>cost_of_not_doing</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G127" t="n">
@@ -23938,16 +23935,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Related / Overlaps With (Initiative IDs)</t>
+          <t>Cost of Not Doing (strategic risk)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>related_to</t>
+          <t>cost_of_not_doing</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -23966,16 +23963,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Dependencies / Blockers</t>
+          <t>Related / Overlaps With (Initiative IDs)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>dependencies_blockers</t>
+          <t>related_to</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -23994,16 +23991,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Dependencies / Blockers</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>dependencies_blockers</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -24022,16 +24019,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Value Type</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>value_basis</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -24050,16 +24047,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Time to First Revenue (months)</t>
+          <t>Value Basis</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>time_to_first_revenue_months</t>
+          <t>value_basis</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -24078,16 +24075,16 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Primary KR (Metric Name)</t>
+          <t>Time to First Revenue (months)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>kr_metric</t>
+          <t>time_to_first_revenue_months</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -24106,16 +24103,16 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -24134,21 +24131,21 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Artifacts (links)</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>artifacts</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G135" t="n">
@@ -24162,25 +24159,25 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Artifacts (links)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>artifacts</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G136" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -24190,16 +24187,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Spec Status</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>spec_status</t>
+          <t>documents</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -24218,25 +24215,25 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Spec Status</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>product_manager</t>
+          <t>spec_status</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G138" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="139">
@@ -24246,16 +24243,16 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>designer</t>
+          <t>product_manager</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -24274,16 +24271,16 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>designer</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -24302,16 +24299,16 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Business Manager</t>
+          <t>Analyst</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>business_manager</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -24330,21 +24327,21 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>AI Draft (needs review)</t>
+          <t>Business Manager</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>ai_draft</t>
+          <t>business_manager</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G142" t="n">
@@ -24354,39 +24351,29 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Timeline</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+          <t>Discovery</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>AI Draft (needs review)</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>ai_draft</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G143" t="n">
         <v>1</v>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="144">
@@ -24395,17 +24382,22 @@
           <t>Timeline</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+        </is>
+      </c>
       <c r="C144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -24429,16 +24421,16 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -24462,16 +24454,16 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -24481,6 +24473,11 @@
       </c>
       <c r="G146" t="n">
         <v>1</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="147">
@@ -24490,25 +24487,25 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Days in Current Phase</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>days_in_phase</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G147" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -24518,25 +24515,25 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Days in Current Phase</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>days_in_phase</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149">
@@ -24546,16 +24543,16 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Start Discovery</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>start_discovery</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -24574,16 +24571,16 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Start Definition</t>
+          <t>Start Discovery</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>start_definition</t>
+          <t>start_discovery</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -24602,16 +24599,16 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Start Building</t>
+          <t>Start Definition</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>start_building</t>
+          <t>start_definition</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -24630,16 +24627,16 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Start Beta-Test</t>
+          <t>Start Building</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>start_beta</t>
+          <t>start_building</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -24658,16 +24655,16 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Start Experiment</t>
+          <t>Start Beta-Test</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>start_experiment</t>
+          <t>start_beta</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -24686,16 +24683,16 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Start Roll-Out</t>
+          <t>Start Experiment</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>start_rollout</t>
+          <t>start_experiment</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -24714,16 +24711,16 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>G2M Date (actual)</t>
+          <t>Start Roll-Out</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>g2m_date_actual</t>
+          <t>start_rollout</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -24742,25 +24739,25 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Discovery Time (days)</t>
+          <t>G2M Date (actual)</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>time_discovery_days</t>
+          <t>g2m_date_actual</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G156" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157">
@@ -24770,16 +24767,16 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Definition Time (days)</t>
+          <t>Discovery Time (days)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>time_definition_days</t>
+          <t>time_discovery_days</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -24798,16 +24795,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Building Time (days)</t>
+          <t>Definition Time (days)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>time_building_days</t>
+          <t>time_definition_days</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -24826,16 +24823,16 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Beta-Test Time (days)</t>
+          <t>Building Time (days)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>time_beta_days</t>
+          <t>time_building_days</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -24854,16 +24851,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Experiment Time (days)</t>
+          <t>Beta-Test Time (days)</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>time_experiment_days</t>
+          <t>time_beta_days</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -24882,16 +24879,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Roll-Out Time (days)</t>
+          <t>Experiment Time (days)</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>time_rollout_days</t>
+          <t>time_experiment_days</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -24910,16 +24907,16 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Time to Market (days)</t>
+          <t>Roll-Out Time (days)</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>time_to_market_days</t>
+          <t>time_rollout_days</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -24938,16 +24935,16 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Actual Build (weeks)</t>
+          <t>Time to Market (days)</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>actual_build_weeks</t>
+          <t>time_to_market_days</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -24966,16 +24963,16 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Build vs Estimate High (%)</t>
+          <t>Actual Build (weeks)</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>build_vs_estimate_high_pct</t>
+          <t>actual_build_weeks</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -24994,16 +24991,16 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Blocked Days</t>
+          <t>Build vs Estimate High (%)</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>blocked_days</t>
+          <t>build_vs_estimate_high_pct</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -25018,39 +25015,29 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>History</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Blocked Days</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>blocked_days</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G166" t="n">
-        <v>1</v>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="167">
@@ -25059,17 +25046,22 @@
           <t>History</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+        </is>
+      </c>
       <c r="C167" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -25093,16 +25085,16 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -25126,16 +25118,16 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>initiative_status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -25145,6 +25137,11 @@
       </c>
       <c r="G169" t="n">
         <v>1</v>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="170">
@@ -25154,16 +25151,16 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Build Status</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -25172,7 +25169,7 @@
         </is>
       </c>
       <c r="G170" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171">
@@ -25182,16 +25179,16 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -25200,7 +25197,7 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172">
@@ -25210,16 +25207,16 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -25238,21 +25235,21 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G173" t="n">
@@ -25266,16 +25263,16 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Decided By</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>decided_by</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -25294,16 +25291,16 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Decision Date</t>
+          <t>Decided By</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>decision_date</t>
+          <t>decided_by</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -25322,21 +25319,21 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Status Changed At</t>
+          <t>Decision Date</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>status_changed_at</t>
+          <t>decision_date</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G176" t="n">
@@ -25350,16 +25347,16 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Phase Changed At</t>
+          <t>Status Changed At</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>phase_changed_at</t>
+          <t>status_changed_at</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -25378,21 +25375,21 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>Phase Changed At</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>last_edited_at</t>
+          <t>phase_changed_at</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G178" t="n">
@@ -25406,21 +25403,21 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Last Edited By</t>
+          <t>Last Updated</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>last_edited_by</t>
+          <t>last_edited_at</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G179" t="n">
@@ -25434,16 +25431,16 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Created At</t>
+          <t>Last Edited By</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>last_edited_by</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -25462,16 +25459,16 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Created By</t>
+          <t>Created At</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -25490,16 +25487,16 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Created Via</t>
+          <t>Created By</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>created_via</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -25518,16 +25515,16 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Last Reviewed</t>
+          <t>Created Via</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>last_reviewed_at</t>
+          <t>created_via</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -25546,16 +25543,16 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Review Overdue</t>
+          <t>Last Reviewed</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>review_overdue</t>
+          <t>last_reviewed_at</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -25564,7 +25561,7 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185">
@@ -25574,16 +25571,16 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Item Age (days)</t>
+          <t>Review Overdue</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>item_age_days</t>
+          <t>review_overdue</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -25602,16 +25599,16 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Archived</t>
+          <t>Item Age (days)</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>item_age_days</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -25620,45 +25617,35 @@
         </is>
       </c>
       <c r="G186" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Cycle review</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>archived</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G187" t="n">
         <v>1</v>
-      </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="188">
@@ -25667,17 +25654,22 @@
           <t>Cycle review</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+        </is>
+      </c>
       <c r="C188" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -25701,16 +25693,16 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -25734,16 +25726,16 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -25753,6 +25745,11 @@
       </c>
       <c r="G190" t="n">
         <v>1</v>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="191">
@@ -25762,25 +25759,25 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G191" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -25790,16 +25787,16 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -25818,16 +25815,16 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Candidate Tag</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>candidate_tag</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -25846,16 +25843,16 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Deferred Count</t>
+          <t>Candidate Tag</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>deferred_count</t>
+          <t>candidate_tag</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -25874,16 +25871,16 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Deferral Reason</t>
+          <t>Deferred Count</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>deferral_reason</t>
+          <t>deferred_count</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -25902,16 +25899,16 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Added After Commit</t>
+          <t>Deferral Reason</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>added_after_commit</t>
+          <t>deferral_reason</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -25930,25 +25927,25 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Added After Commit</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>added_after_commit</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G197" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="198">
@@ -25958,21 +25955,21 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G198" t="n">
@@ -25986,16 +25983,16 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -26004,7 +26001,7 @@
         </is>
       </c>
       <c r="G199" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="200">
@@ -26014,16 +26011,16 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>MoSCoW</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>moscow</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -26032,7 +26029,7 @@
         </is>
       </c>
       <c r="G200" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="201">
@@ -26042,24 +26039,52 @@
         </is>
       </c>
       <c r="C201" t="n">
+        <v>14</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>MoSCoW</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>moscow</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G201" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
         <v>15</v>
       </c>
-      <c r="D201" t="inlineStr">
+      <c r="D202" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
+      <c r="E202" t="inlineStr">
         <is>
           <t>decision</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr">
+      <c r="F202" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="G201" t="n">
+      <c r="G202" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Release 0.47.0: Business Value wording, item panel width and search, land on last screen (R-112)
Rename Value Type, Value (EUR, 12-month run-rate) and Value Basis to Business Value Type (five values), Business Value (12m run-rate, organization currency) and Business Value Basis (migration 0053). Item panel: tidy header, drag-to-resize width saved in the user profile, field search. Last screen and view saved per account and restored on sign-in.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMdyHtUDStUhNdNnj8JmdE
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -2272,7 +2272,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Business Value Type</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -2287,12 +2287,12 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Incremental revenue · Defend existing revenue · Save money / operational efficiency</t>
+          <t>New revenue · Increase revenue · Defend revenue · Decrease costs · Other</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Always one of: Incremental revenue, Defend existing revenue, Save money / operational efficiency</t>
+          <t>Always one of: New revenue, Increase revenue, Defend revenue, Decrease costs, Other</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -2352,7 +2352,7 @@
       <c r="F26" s="9" t="inlineStr"/>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Single universal value in EUR as a 12-month run-rate, comparable across all initiatives for stack ranking</t>
+          <t>Single universal value in the organization currency as a 12-month run-rate, comparable across all initiatives for stack ranking</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Business Value Basis</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -5588,7 +5588,7 @@
       </c>
       <c r="K79" s="9" t="inlineStr">
         <is>
-          <t>Show only when Value Type = Save money.</t>
+          <t>Show only when Business Value Type = Save money.</t>
         </is>
       </c>
       <c r="L79" s="9" t="inlineStr"/>
@@ -6238,7 +6238,7 @@
       </c>
       <c r="K89" s="9" t="inlineStr">
         <is>
-          <t>Mirrors Value Basis. Weighted value per build-week is only as good as the estimate.</t>
+          <t>Mirrors Business Value Basis. Weighted value per build-week is only as good as the estimate.</t>
         </is>
       </c>
       <c r="L89" s="9" t="inlineStr"/>
@@ -12699,7 +12699,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Business Value Type</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -12737,7 +12737,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Business Value Basis</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -19682,7 +19682,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Business Value Basis</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -19727,7 +19727,7 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Business Value Type</t>
         </is>
       </c>
     </row>
@@ -19810,7 +19810,7 @@
       </c>
       <c r="Q2" s="15" t="inlineStr">
         <is>
-          <t>Incremental revenue</t>
+          <t>New revenue</t>
         </is>
       </c>
     </row>
@@ -19893,7 +19893,7 @@
       </c>
       <c r="Q3" s="15" t="inlineStr">
         <is>
-          <t>Defend existing revenue</t>
+          <t>Increase revenue</t>
         </is>
       </c>
     </row>
@@ -19972,7 +19972,7 @@
       </c>
       <c r="Q4" s="15" t="inlineStr">
         <is>
-          <t>Save money / operational efficiency</t>
+          <t>Defend revenue</t>
         </is>
       </c>
     </row>
@@ -20039,7 +20039,11 @@
           <t>Not yet decided</t>
         </is>
       </c>
-      <c r="Q5" s="15" t="n"/>
+      <c r="Q5" s="15" t="inlineStr">
+        <is>
+          <t>Decrease costs</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -20084,7 +20088,11 @@
         </is>
       </c>
       <c r="P6" s="15" t="n"/>
-      <c r="Q6" s="15" t="n"/>
+      <c r="Q6" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -20543,7 +20551,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -22919,7 +22927,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -23443,7 +23451,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Value (EUR, 12-month run-rate)</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -24023,7 +24031,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Value Type</t>
+          <t>Business Value Type</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -24051,7 +24059,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Value Basis</t>
+          <t>Business Value Basis</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">

</xml_diff>

<commit_message>
Planned Quarter: G2M Quarter becomes a field people set (R-114, release 0.50.0)
Stored g2m_quarter column (migration 0057, backfilled once from G2M Date), calendar quarters only,
generated list plus quarters in use, panel/grid/bulk/import/MCP editing, mismatch warning, tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMdyHsakKNjXejMW7hthwG
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -3452,7 +3452,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Planned Quarter</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -3462,43 +3462,43 @@
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Computed</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr"/>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>Go-to-market quarter</t>
+          <t>Calendar quarter the work is planned for, chosen by a person</t>
         </is>
       </c>
       <c r="H44" s="9" t="inlineStr">
         <is>
-          <t>After dates are known</t>
+          <t>When planning</t>
         </is>
       </c>
       <c r="I44" s="9" t="inlineStr">
         <is>
-          <t>Computed</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="J44" s="10" t="inlineStr">
         <is>
-          <t>Auto-derive</t>
+          <t>Modify (R-114)</t>
         </is>
       </c>
       <c r="K44" s="9" t="inlineStr">
         <is>
-          <t>Derived from G2M Date (actual, else est), e.g. 2026-Q4. Manual input only while no date exists.</t>
+          <t>Was calculated from G2M Date; since R-114 a person sets it (Q1 to Q4 plus year, calendar quarters only). The list is generated: previous year to next 3 years, plus any value in use. Independent of G2M Date (est); a date outside the quarter shows a hint.</t>
         </is>
       </c>
       <c r="L44" s="9" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>Computed (view or function, not stored)</t>
+          <t>Column on items</t>
         </is>
       </c>
       <c r="N44" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -13441,7 +13441,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Planned Quarter</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -13456,12 +13456,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Computed</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Computed (read-only)</t>
+          <t>Editable</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -18436,7 +18436,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167"/>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>
@@ -19575,7 +19574,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>#48 G2M Quarter</t>
+          <t>#48 Planned Quarter (was G2M Quarter)</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -22151,7 +22150,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Planned Quarter</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -23395,7 +23394,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>G2M Quarter</t>
+          <t>Planned Quarter</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">

</xml_diff>

<commit_message>
Focus Area and Audience become open lists with suggestions (issue #246)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMdyHtfXpzoTRtwG2JPTAU
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -1277,11 +1277,7 @@
           <t>Select</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Formats · Demand/Optimisation · Publishers</t>
-        </is>
-      </c>
+      <c r="F9" s="9" t="n"/>
       <c r="G9" s="9" t="inlineStr">
         <is>
           <t>Formats, Demand/Optimisation, Publishers, Backlog (as in v1)</t>
@@ -4133,11 +4129,7 @@
           <t>Select</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
-        <is>
-          <t>Publishers · Demand partners · Brands and agencies · Internal · Mixed</t>
-        </is>
-      </c>
+      <c r="F55" s="9" t="n"/>
       <c r="G55" s="9" t="inlineStr">
         <is>
           <t>Publishers, Demand partners, Brands and agencies, Internal, Mixed</t>

</xml_diff>

<commit_message>
Status alignment step 2: new Build, Initiative and Planning Status values, migration and tests (issue #247)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMdyHqJM3LRrraf38KTreW
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -955,7 +955,7 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Backlog · Not Started · In Progress · Paused · Completed · Cancelled</t>
+          <t>Not started · In progress · Done · Cancelled</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>GitHub -&gt; app. Tracking issue closed as completed -&gt; Status Completed; closed as not planned -&gt; Cancelled; first child issue in progress -&gt; In Progress. Applied automatically, audit-logged.</t>
+          <t>GitHub -&gt; app, read-only. Fixed vocabulary shared with Jira: tracking issue closed as completed -&gt; Done; closed as not planned -&gt; Cancelled; reopened -&gt; Not started; first child issue in progress -&gt; In progress. Counts from Gate B (Define to Build) onward. Applied automatically, audit-logged.</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
@@ -9899,12 +9899,12 @@
       </c>
       <c r="F146" s="9" t="inlineStr">
         <is>
-          <t>Candidate · Included · Committed · Deferred · Dropped</t>
+          <t>Backlog · Not started · Candidate · Included · Committed · Deferred · Dropped</t>
         </is>
       </c>
       <c r="G146" s="9" t="inlineStr">
         <is>
-          <t>Where the item stands in the planning cycle.</t>
+          <t>Where the item stands before and during planning: Backlog and Not started first, then the planning cycle (Candidate to Dropped).</t>
         </is>
       </c>
       <c r="H146" s="9" t="inlineStr">
@@ -9938,7 +9938,7 @@
         </is>
       </c>
       <c r="N146" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -11341,12 +11341,12 @@
       </c>
       <c r="F167" s="9" t="inlineStr">
         <is>
-          <t>Backlog · Not Started · In Progress · Paused · Completed · Cancelled</t>
+          <t>Active · On hold · Cancelled</t>
         </is>
       </c>
       <c r="G167" s="9" t="inlineStr">
         <is>
-          <t>Where the initiative itself stands, set by people (a closed GitHub or Jira ticket only means the build is complete: see Build Status).</t>
+          <t>Whether the initiative is alive, set by people: Active, On hold or Cancelled. Completed and Sunset come from Initiative Phase; Backlog and Not started are Planning Status. A closed GitHub or Jira ticket only means the build is done: see Build Status.</t>
         </is>
       </c>
       <c r="H167" s="9" t="inlineStr">
@@ -17597,8 +17597,18 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P146" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="147">
@@ -18436,6 +18446,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>
@@ -18467,6 +18478,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J168" t="inlineStr">
         <is>
           <t>Y</t>
@@ -18478,7 +18494,7 @@
         </is>
       </c>
       <c r="P168" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="169">
@@ -20212,7 +20228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -20962,21 +20978,21 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -21486,17 +21502,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>initiative_status</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -21570,12 +21586,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Delivery Status</t>
+          <t>Last Synced</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>gh_project_status</t>
+          <t>last_synced</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -21598,12 +21614,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Last Synced</t>
+          <t>Synced With</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>last_synced</t>
+          <t>synced_with</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -21626,17 +21642,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Synced With</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>synced_with</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G48" t="n">
@@ -21654,21 +21670,21 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -21682,12 +21698,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Schedule Variance (pp)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>schedule_variance_pp</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -21710,21 +21726,21 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Schedule Variance (pp)</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>schedule_variance_pp</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -21738,12 +21754,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -21752,7 +21768,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -21766,21 +21782,21 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>Blocked Issues (#)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>blocked_issues</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
@@ -21794,12 +21810,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Blocked Issues (#)</t>
+          <t>Stale Issues (#)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>blocked_issues</t>
+          <t>stale_issues</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -21822,12 +21838,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Stale Issues (#)</t>
+          <t>Scope Added (#)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>stale_issues</t>
+          <t>scope_added</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -21850,12 +21866,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Scope Added (#)</t>
+          <t>Open PRs (#)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>scope_added</t>
+          <t>open_prs</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -21878,12 +21894,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Open PRs (#)</t>
+          <t>CI Status</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>open_prs</t>
+          <t>ci_status</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -21906,12 +21922,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>CI Status</t>
+          <t>Assignees</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ci_status</t>
+          <t>assignees</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -21934,12 +21950,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Assignees</t>
+          <t>Breakdown Status</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>assignees</t>
+          <t>breakdown_status</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -21948,35 +21964,45 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Go-to-market</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Breakdown Status</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>breakdown_status</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -21985,22 +22011,17 @@
           <t>Go-to-market</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
-        </is>
-      </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -22024,16 +22045,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -22057,16 +22078,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -22076,11 +22097,6 @@
       </c>
       <c r="G63" t="n">
         <v>1</v>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="64">
@@ -22090,21 +22106,21 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Audience</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>audience</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G64" t="n">
@@ -22118,25 +22134,25 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Audience</t>
+          <t>Planned Quarter</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
@@ -22146,16 +22162,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Planned Quarter</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -22164,7 +22180,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -22174,16 +22190,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Date Precision</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>date_precision</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -22202,21 +22218,21 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Date Precision</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>date_precision</t>
+          <t>target_scope</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -22230,16 +22246,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Target Markets</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>target_scope</t>
+          <t>live_scope</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -22258,21 +22274,21 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Live Markets</t>
+          <t>Target Segments (customer-safe)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>live_scope</t>
+          <t>target_segments</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G70" t="n">
@@ -22286,21 +22302,21 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Target Segments (customer-safe)</t>
+          <t>Target Customers (#)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>target_segments</t>
+          <t>target_customers</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G71" t="n">
@@ -22314,16 +22330,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Target Customers (#)</t>
+          <t>Customers Live (#)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>target_customers</t>
+          <t>customers_live</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -22332,7 +22348,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73">
@@ -22342,16 +22358,16 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Customers Live (#)</t>
+          <t>Roll-out %</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>customers_live</t>
+          <t>rollout_pct</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -22370,16 +22386,16 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Roll-out %</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>rollout_pct</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -22398,25 +22414,25 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Value Proposition (customer-safe)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>value_proposition</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G75" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -22426,16 +22442,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Value Proposition (customer-safe)</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>value_proposition</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -22454,21 +22470,21 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>GTM / Enablement Notes</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>gtm_enablement_notes</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G77" t="n">
@@ -22482,21 +22498,21 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GTM / Enablement Notes</t>
+          <t>Screenshots</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>gtm_enablement_notes</t>
+          <t>screenshots</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G78" t="n">
@@ -22506,20 +22522,25 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Outcomes</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Screenshots</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>screenshots</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -22529,6 +22550,11 @@
       </c>
       <c r="G79" t="n">
         <v>1</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -22537,22 +22563,17 @@
           <t>Outcomes</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
-        </is>
-      </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -22576,16 +22597,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -22609,16 +22630,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -22628,11 +22649,6 @@
       </c>
       <c r="G82" t="n">
         <v>1</v>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="83">
@@ -22642,25 +22658,25 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Outcome Status</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>outcome_status</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G83" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="84">
@@ -22670,16 +22686,16 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Outcome Status</t>
+          <t>Outcome Review Date</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>outcome_status</t>
+          <t>outcome_review_date</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -22698,25 +22714,25 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Outcome Review Date</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>outcome_review_date</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G85" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -22726,16 +22742,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Primary KR (Metric Name)</t>
+          <t>Primary KR Unit</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>kr_metric</t>
+          <t>kr_unit</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -22754,16 +22770,16 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Primary KR Unit</t>
+          <t>Primary KR Start Value</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>kr_unit</t>
+          <t>kr_start</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -22782,16 +22798,16 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Primary KR Start Value</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>kr_start</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -22810,25 +22826,25 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Realized KR Value</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>realized_kr_value</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90">
@@ -22838,16 +22854,16 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Realized KR Value</t>
+          <t>% Realized KR Value</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>realized_kr_value</t>
+          <t>kr_realized_pct</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -22866,21 +22882,21 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>% Realized KR Value</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>kr_realized_pct</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G91" t="n">
@@ -22894,25 +22910,25 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G92" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -22922,25 +22938,25 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Business Value (12m run-rate)</t>
+          <t>Realized EUR per year</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>realized_per_year</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G93" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="94">
@@ -22950,16 +22966,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Realized EUR per year</t>
+          <t>Value vs Prediction (%)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>realized_per_year</t>
+          <t>value_variance_pct</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -22978,16 +22994,16 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Value vs Prediction (%)</t>
+          <t>Outcome Verdict</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>value_variance_pct</t>
+          <t>outcome_verdict</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -23006,16 +23022,16 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Outcome Verdict</t>
+          <t>Time to First Use (days)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>outcome_verdict</t>
+          <t>time_to_first_use_days</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -23034,16 +23050,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Time to First Use (days)</t>
+          <t>Retention (%)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>time_to_first_use_days</t>
+          <t>retention_pct</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -23062,16 +23078,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Retention (%)</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>retention_pct</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -23086,29 +23102,39 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Leadership</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G99" t="n">
-        <v>7</v>
+        <v>1</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -23117,22 +23143,17 @@
           <t>Leadership</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
-        </is>
-      </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -23156,16 +23177,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -23189,16 +23210,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -23208,11 +23229,6 @@
       </c>
       <c r="G102" t="n">
         <v>1</v>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="103">
@@ -23222,16 +23238,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Group</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -23250,16 +23266,16 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Initiative Group</t>
+          <t>Roadmap Category</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>roadmap_category</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -23278,16 +23294,16 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Roadmap Category</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>roadmap_category</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -23306,16 +23322,16 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -23334,25 +23350,25 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108">
@@ -23362,25 +23378,25 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Planned Quarter</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -23390,16 +23406,16 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Planned Quarter</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -23418,25 +23434,25 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G110" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -23446,16 +23462,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Business Value (12m run-rate)</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -23474,21 +23490,21 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G112" t="n">
@@ -23502,25 +23518,25 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Current Gate</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>current_gate</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Gates</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114">
@@ -23530,25 +23546,25 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Current Gate</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>current_gate</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Gates</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="115">
@@ -23558,25 +23574,25 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>sponsor</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -23586,21 +23602,21 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Next Review Date</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>sponsor</t>
+          <t>next_review_date</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G116" t="n">
@@ -23614,21 +23630,21 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Next Review Date</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>next_review_date</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G117" t="n">
@@ -23638,20 +23654,25 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Leadership</t>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -23661,6 +23682,11 @@
       </c>
       <c r="G118" t="n">
         <v>1</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -23669,22 +23695,17 @@
           <t>Discovery</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
-        </is>
-      </c>
       <c r="C119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -23708,16 +23729,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -23741,16 +23762,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -23760,11 +23781,6 @@
       </c>
       <c r="G121" t="n">
         <v>1</v>
-      </c>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="122">
@@ -23774,16 +23790,16 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Change Type</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>change_type</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -23802,16 +23818,16 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Change Type</t>
+          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>change_type</t>
+          <t>hypothesis</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -23830,21 +23846,21 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
+          <t>Request Origin</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>hypothesis</t>
+          <t>request_origin</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -23858,16 +23874,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Request Origin</t>
+          <t>Customers Requesting (#)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>request_origin</t>
+          <t>customers_requesting</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -23886,21 +23902,21 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Customers Requesting (#)</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>customers_requesting</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G126" t="n">
@@ -23914,21 +23930,21 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Cost of Not Doing (strategic risk)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>cost_of_not_doing</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G127" t="n">
@@ -23942,16 +23958,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Cost of Not Doing (strategic risk)</t>
+          <t>Related / Overlaps With (Initiative IDs)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>cost_of_not_doing</t>
+          <t>related_to</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -23970,16 +23986,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Related / Overlaps With (Initiative IDs)</t>
+          <t>Dependencies / Blockers</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>related_to</t>
+          <t>dependencies_blockers</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -23998,16 +24014,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Dependencies / Blockers</t>
+          <t>Business Value Type</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>dependencies_blockers</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -24026,16 +24042,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Business Value Type</t>
+          <t>Business Value Basis</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>value_basis</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -24054,16 +24070,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Business Value Basis</t>
+          <t>Time to First Revenue (months)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>value_basis</t>
+          <t>time_to_first_revenue_months</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -24082,16 +24098,16 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Time to First Revenue (months)</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>time_to_first_revenue_months</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -24110,16 +24126,16 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Primary KR (Metric Name)</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>kr_metric</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -24138,21 +24154,21 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Artifacts (links)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>artifacts</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G135" t="n">
@@ -24166,25 +24182,25 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Artifacts (links)</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>artifacts</t>
+          <t>documents</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G136" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="137">
@@ -24194,16 +24210,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Spec Status</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>spec_status</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -24222,25 +24238,25 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Spec Status</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>spec_status</t>
+          <t>product_manager</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G138" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -24250,16 +24266,16 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>product_manager</t>
+          <t>designer</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -24278,16 +24294,16 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Analyst</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>designer</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -24306,16 +24322,16 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Business Manager</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>business_manager</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -24334,21 +24350,21 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Business Manager</t>
+          <t>AI Draft (needs review)</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>business_manager</t>
+          <t>ai_draft</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G142" t="n">
@@ -24358,29 +24374,39 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Discovery</t>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>AI Draft (needs review)</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>ai_draft</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G143" t="n">
         <v>1</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="144">
@@ -24389,22 +24415,17 @@
           <t>Timeline</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
-        </is>
-      </c>
       <c r="C144" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -24428,16 +24449,16 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -24461,16 +24482,16 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -24480,11 +24501,6 @@
       </c>
       <c r="G146" t="n">
         <v>1</v>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="147">
@@ -24494,25 +24510,25 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Days in Current Phase</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>days_in_phase</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148">
@@ -24522,25 +24538,25 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Days in Current Phase</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>days_in_phase</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G148" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -24550,16 +24566,16 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Start Discovery</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>start_discovery</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -24578,16 +24594,16 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Start Discovery</t>
+          <t>Start Definition</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>start_discovery</t>
+          <t>start_definition</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -24606,16 +24622,16 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Start Definition</t>
+          <t>Start Building</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>start_definition</t>
+          <t>start_building</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -24634,16 +24650,16 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Start Building</t>
+          <t>Start Beta-Test</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>start_building</t>
+          <t>start_beta</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -24662,16 +24678,16 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Start Beta-Test</t>
+          <t>Start Experiment</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>start_beta</t>
+          <t>start_experiment</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -24690,16 +24706,16 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Start Experiment</t>
+          <t>Start Roll-Out</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>start_experiment</t>
+          <t>start_rollout</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -24718,16 +24734,16 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Start Roll-Out</t>
+          <t>G2M Date (actual)</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>start_rollout</t>
+          <t>g2m_date_actual</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -24746,25 +24762,25 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>G2M Date (actual)</t>
+          <t>Discovery Time (days)</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>g2m_date_actual</t>
+          <t>time_discovery_days</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G156" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="157">
@@ -24774,16 +24790,16 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Discovery Time (days)</t>
+          <t>Definition Time (days)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>time_discovery_days</t>
+          <t>time_definition_days</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -24802,16 +24818,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Definition Time (days)</t>
+          <t>Building Time (days)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>time_definition_days</t>
+          <t>time_building_days</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -24830,16 +24846,16 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Building Time (days)</t>
+          <t>Beta-Test Time (days)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>time_building_days</t>
+          <t>time_beta_days</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -24858,16 +24874,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Beta-Test Time (days)</t>
+          <t>Experiment Time (days)</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>time_beta_days</t>
+          <t>time_experiment_days</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -24886,16 +24902,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Experiment Time (days)</t>
+          <t>Roll-Out Time (days)</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>time_experiment_days</t>
+          <t>time_rollout_days</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -24914,16 +24930,16 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Roll-Out Time (days)</t>
+          <t>Time to Market (days)</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>time_rollout_days</t>
+          <t>time_to_market_days</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -24942,16 +24958,16 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Time to Market (days)</t>
+          <t>Actual Build (weeks)</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>time_to_market_days</t>
+          <t>actual_build_weeks</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -24970,16 +24986,16 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Actual Build (weeks)</t>
+          <t>Build vs Estimate High (%)</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>actual_build_weeks</t>
+          <t>build_vs_estimate_high_pct</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -24998,16 +25014,16 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Build vs Estimate High (%)</t>
+          <t>Blocked Days</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>build_vs_estimate_high_pct</t>
+          <t>blocked_days</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -25022,29 +25038,39 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Timeline</t>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Blocked Days</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>blocked_days</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G166" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="167">
@@ -25053,22 +25079,17 @@
           <t>History</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
-        </is>
-      </c>
       <c r="C167" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -25092,16 +25113,16 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -25125,30 +25146,25 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G169" t="n">
         <v>1</v>
-      </c>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="170">
@@ -25158,16 +25174,16 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>initiative_status</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -25176,7 +25192,7 @@
         </is>
       </c>
       <c r="G170" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171">
@@ -25186,16 +25202,16 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Build Status</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -25204,7 +25220,7 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172">
@@ -25214,16 +25230,16 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -25242,21 +25258,21 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G173" t="n">
@@ -25270,16 +25286,16 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Decided By</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>decided_by</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -25298,16 +25314,16 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Decided By</t>
+          <t>Decision Date</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>decided_by</t>
+          <t>decision_date</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -25326,21 +25342,21 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Decision Date</t>
+          <t>Status Changed At</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>decision_date</t>
+          <t>status_changed_at</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G176" t="n">
@@ -25354,16 +25370,16 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Status Changed At</t>
+          <t>Phase Changed At</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>status_changed_at</t>
+          <t>phase_changed_at</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -25382,21 +25398,21 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Phase Changed At</t>
+          <t>Last Updated</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>phase_changed_at</t>
+          <t>last_edited_at</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G178" t="n">
@@ -25410,21 +25426,21 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>Last Edited By</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>last_edited_at</t>
+          <t>last_edited_by</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G179" t="n">
@@ -25438,16 +25454,16 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Last Edited By</t>
+          <t>Created At</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>last_edited_by</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -25466,16 +25482,16 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Created At</t>
+          <t>Created By</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -25494,16 +25510,16 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Created By</t>
+          <t>Created Via</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>created_via</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -25522,16 +25538,16 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Created Via</t>
+          <t>Last Reviewed</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>created_via</t>
+          <t>last_reviewed_at</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -25550,16 +25566,16 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Last Reviewed</t>
+          <t>Review Overdue</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>last_reviewed_at</t>
+          <t>review_overdue</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -25568,7 +25584,7 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="185">
@@ -25578,16 +25594,16 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Review Overdue</t>
+          <t>Item Age (days)</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>review_overdue</t>
+          <t>item_age_days</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -25606,16 +25622,16 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Item Age (days)</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>item_age_days</t>
+          <t>archived</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -25624,35 +25640,45 @@
         </is>
       </c>
       <c r="G186" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Archived</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G187" t="n">
         <v>1</v>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="188">
@@ -25661,22 +25687,17 @@
           <t>Cycle review</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
-        </is>
-      </c>
       <c r="C188" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -25700,16 +25721,16 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -25733,16 +25754,16 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -25752,11 +25773,6 @@
       </c>
       <c r="G190" t="n">
         <v>1</v>
-      </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="191">
@@ -25766,16 +25782,16 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -25794,16 +25810,16 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -25822,16 +25838,16 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Candidate Tag</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>candidate_tag</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -25850,16 +25866,16 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Candidate Tag</t>
+          <t>Deferred Count</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>candidate_tag</t>
+          <t>deferred_count</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -25878,16 +25894,16 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Deferred Count</t>
+          <t>Deferral Reason</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>deferred_count</t>
+          <t>deferral_reason</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -25906,16 +25922,16 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Deferral Reason</t>
+          <t>Added After Commit</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>deferral_reason</t>
+          <t>added_after_commit</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -25934,25 +25950,25 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Added After Commit</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>added_after_commit</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G197" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198">
@@ -25962,21 +25978,21 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G198" t="n">
@@ -25990,16 +26006,16 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -26008,7 +26024,7 @@
         </is>
       </c>
       <c r="G199" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="200">
@@ -26018,16 +26034,16 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>MoSCoW</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>moscow</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -26036,7 +26052,7 @@
         </is>
       </c>
       <c r="G200" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -26046,52 +26062,24 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>MoSCoW</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>moscow</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G201" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>Cycle review</t>
-        </is>
-      </c>
-      <c r="C202" t="n">
-        <v>15</v>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="E202" t="inlineStr">
-        <is>
-          <t>decision</t>
-        </is>
-      </c>
-      <c r="F202" t="inlineStr">
-        <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="G202" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Initiative Status: Completed again, filled for finished initiatives (issue #247 follow-up)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMdyHqJM3LRrraf38KTreW
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -11333,12 +11333,12 @@
       </c>
       <c r="F167" s="9" t="inlineStr">
         <is>
-          <t>Active · On hold · Cancelled</t>
+          <t>Active · On hold · Completed · Cancelled</t>
         </is>
       </c>
       <c r="G167" s="9" t="inlineStr">
         <is>
-          <t>Whether the initiative is alive, set by people: Active, On hold or Cancelled. Completed and Sunset come from Initiative Phase; Backlog and Not started are Planning Status. A closed GitHub or Jira ticket only means the build is done: see Build Status.</t>
+          <t>Whether the initiative is alive, finished or dead, set by people: Active, On hold, Completed or Cancelled. Initiative Phase says where it is in the lifecycle; Backlog and Not started are Planning Status. A closed GitHub or Jira ticket only means the build is done: see Build Status.</t>
         </is>
       </c>
       <c r="H167" s="9" t="inlineStr">
@@ -18438,7 +18438,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167"/>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add the Tracker Ownership field (N48), Delivery view column and Help (#256)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMdyHpaqSbfVToCQJMHPeK
</commit_message>
<xml_diff>
--- a/docs/reference/Roadmap_v4_field_dictionary.xlsx
+++ b/docs/reference/Roadmap_v4_field_dictionary.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N170"/>
+  <dimension ref="A1:N171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11571,6 +11571,76 @@
         <v>1</v>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>N48</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Delivery (GitHub)</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Tracker Ownership</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>tracker_ownership</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Product Velocity · Tracker (read only)</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Who owns what this linked initiative is. Product Velocity: it sends the name, summary, description and hypothesis to the tracker after a preview and a confirmation. Tracker (read only): it only follows the issue and nothing is sent. Status and progress are the tracker's in both cases.</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>When the initiative is linked to an issue</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>New (2026-10-29)</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Asked for by Ashu (2026-10-29, request 253, issue #256): show who owns a pulled-in or linked item, instead of only in the item panel.</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Not synced: shown from the GitHub link and read-only here. Change it on the item's GitHub tab.</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>Derived in the app from the GitHub link (not stored)</t>
+        </is>
+      </c>
+      <c r="N171" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11583,7 +11653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P173"/>
+  <dimension ref="A1:P174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18438,6 +18508,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>
@@ -18582,12 +18653,44 @@
     <row r="172">
       <c r="B172" t="inlineStr">
         <is>
-          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+          <t>Tracker Ownership</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>tracker_ownership</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Delivery (GitHub)</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Computed (read-only)</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="B173" t="inlineStr">
+        <is>
+          <t>Note: every field is a grid column. Views only choose which columns are shown by default; users can add any column through the Columns picker. Customer-safe = may appear in customer-facing reports. Locked = set by GitHub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="B174" t="inlineStr">
         <is>
           <t>2026-10-23: the view columns (Prioritisation … History) on this sheet are SUPERSEDED by sheet 'Default views (ordered)' and docs/reference/default-views.csv (10 views, each with a reading order). Editing mode and the customer-safe flag on this sheet remain valid. 'In view count' is outdated.</t>
         </is>
@@ -20219,7 +20322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21633,17 +21736,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Tracker Ownership</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>tracker_ownership</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G48" t="n">
@@ -21661,21 +21764,21 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -21689,12 +21792,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Schedule Variance (pp)</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>schedule_variance_pp</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -21717,21 +21820,21 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Schedule Variance (pp)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>schedule_variance_pp</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -21745,12 +21848,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -21759,7 +21862,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -21773,21 +21876,21 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Blocked Issues (#)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>blocked_issues</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -21801,12 +21904,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Stale Issues (#)</t>
+          <t>Blocked Issues (#)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>stale_issues</t>
+          <t>blocked_issues</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -21829,12 +21932,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Scope Added (#)</t>
+          <t>Stale Issues (#)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>scope_added</t>
+          <t>stale_issues</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -21857,12 +21960,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Open PRs (#)</t>
+          <t>Scope Added (#)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>open_prs</t>
+          <t>scope_added</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -21885,12 +21988,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CI Status</t>
+          <t>Open PRs (#)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ci_status</t>
+          <t>open_prs</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -21913,12 +22016,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Assignees</t>
+          <t>CI Status</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>assignees</t>
+          <t>ci_status</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -21941,12 +22044,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Breakdown Status</t>
+          <t>Assignees</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>breakdown_status</t>
+          <t>assignees</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -21955,45 +22058,35 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Breakdown Status</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>breakdown_status</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>1</v>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="61">
@@ -22002,17 +22095,22 @@
           <t>Go-to-market</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Launch readiness: audience, markets, customers, adoption and the customer-safe story.</t>
+        </is>
+      </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -22036,16 +22134,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -22069,16 +22167,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -22088,6 +22186,11 @@
       </c>
       <c r="G63" t="n">
         <v>1</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -22097,21 +22200,21 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Audience</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G64" t="n">
@@ -22125,25 +22228,25 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Planned Quarter</t>
+          <t>Audience</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>audience</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -22153,16 +22256,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>G2M Date (est)</t>
+          <t>Planned Quarter</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>g2m_date_est</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -22171,7 +22274,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67">
@@ -22181,16 +22284,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Date Precision</t>
+          <t>G2M Date (est)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>date_precision</t>
+          <t>g2m_date_est</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -22209,21 +22312,21 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Target Markets</t>
+          <t>Date Precision</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>target_scope</t>
+          <t>date_precision</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -22237,16 +22340,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Live Markets</t>
+          <t>Target Markets</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>live_scope</t>
+          <t>target_scope</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -22265,21 +22368,21 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Target Segments (customer-safe)</t>
+          <t>Live Markets</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>target_segments</t>
+          <t>live_scope</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G70" t="n">
@@ -22293,21 +22396,21 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Target Customers (#)</t>
+          <t>Target Segments (customer-safe)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>target_customers</t>
+          <t>target_segments</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G71" t="n">
@@ -22321,16 +22424,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Customers Live (#)</t>
+          <t>Target Customers (#)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>customers_live</t>
+          <t>target_customers</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -22339,7 +22442,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -22349,16 +22452,16 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Roll-out %</t>
+          <t>Customers Live (#)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>rollout_pct</t>
+          <t>customers_live</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -22377,16 +22480,16 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>Roll-out %</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>rollout_pct</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -22405,25 +22508,25 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Value Proposition (customer-safe)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>value_proposition</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G75" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76">
@@ -22433,16 +22536,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Value Proposition (customer-safe)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>value_proposition</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -22461,21 +22564,21 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>GTM / Enablement Notes</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>gtm_enablement_notes</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G77" t="n">
@@ -22489,21 +22592,21 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Screenshots</t>
+          <t>GTM / Enablement Notes</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>screenshots</t>
+          <t>gtm_enablement_notes</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G78" t="n">
@@ -22513,25 +22616,20 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Outcomes</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Screenshots</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>screenshots</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -22541,11 +22639,6 @@
       </c>
       <c r="G79" t="n">
         <v>1</v>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="80">
@@ -22554,17 +22647,22 @@
           <t>Outcomes</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Did it work: key results, adoption, predicted vs realised value and what we learned.</t>
+        </is>
+      </c>
       <c r="C80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -22588,16 +22686,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -22621,16 +22719,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -22640,6 +22738,11 @@
       </c>
       <c r="G82" t="n">
         <v>1</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -22649,25 +22752,25 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Outcome Status</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>outcome_status</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G83" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -22677,16 +22780,16 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Outcome Review Date</t>
+          <t>Outcome Status</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>outcome_review_date</t>
+          <t>outcome_status</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -22705,25 +22808,25 @@
         </is>
       </c>
       <c r="C85" t="n">
+        <v>6</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Outcome Review Date</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>outcome_review_date</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Outcomes</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
         <v>7</v>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Primary KR (Metric Name)</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>kr_metric</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="G85" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -22733,16 +22836,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Primary KR Unit</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>kr_unit</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -22761,16 +22864,16 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Primary KR Start Value</t>
+          <t>Primary KR Unit</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>kr_start</t>
+          <t>kr_unit</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -22789,16 +22892,16 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR Start Value</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_start</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -22817,25 +22920,25 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Realized KR Value</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>realized_kr_value</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -22845,16 +22948,16 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>% Realized KR Value</t>
+          <t>Realized KR Value</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>kr_realized_pct</t>
+          <t>realized_kr_value</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -22873,21 +22976,21 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>% Adoption (live / target customers)</t>
+          <t>% Realized KR Value</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>adoption_pct</t>
+          <t>kr_realized_pct</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Go-to-market</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G91" t="n">
@@ -22901,25 +23004,25 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Business Value (12m run-rate)</t>
+          <t>% Adoption (live / target customers)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>adoption_pct</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Go-to-market</t>
         </is>
       </c>
       <c r="G92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="93">
@@ -22929,25 +23032,25 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Realized EUR per year</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>realized_per_year</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G93" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -22957,16 +23060,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Value vs Prediction (%)</t>
+          <t>Realized EUR per year</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>value_variance_pct</t>
+          <t>realized_per_year</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -22985,16 +23088,16 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Outcome Verdict</t>
+          <t>Value vs Prediction (%)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>outcome_verdict</t>
+          <t>value_variance_pct</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -23013,16 +23116,16 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Time to First Use (days)</t>
+          <t>Outcome Verdict</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>time_to_first_use_days</t>
+          <t>outcome_verdict</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -23041,16 +23144,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Retention (%)</t>
+          <t>Time to First Use (days)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>retention_pct</t>
+          <t>time_to_first_use_days</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -23069,16 +23172,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Retention (%)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>retention_pct</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -23093,39 +23196,29 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Leadership</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="G99" t="n">
-        <v>1</v>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="100">
@@ -23134,17 +23227,22 @@
           <t>Leadership</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Portfolio at a glance: what, where, health, progress, dates, value and decisions.</t>
+        </is>
+      </c>
       <c r="C100" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -23168,16 +23266,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -23201,16 +23299,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -23220,6 +23318,11 @@
       </c>
       <c r="G102" t="n">
         <v>1</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -23229,16 +23332,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Initiative Group</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -23257,16 +23360,16 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Roadmap Category</t>
+          <t>Initiative Group</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>roadmap_category</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -23285,16 +23388,16 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Roadmap Category</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>roadmap_category</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -23313,16 +23416,16 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -23341,25 +23444,25 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Delivery Progress %</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>delivery_progress_pct</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Delivery (GitHub)</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -23369,25 +23472,25 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Planned Quarter</t>
+          <t>Delivery Progress %</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>g2m_quarter</t>
+          <t>delivery_progress_pct</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Delivery (GitHub)</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="109">
@@ -23397,16 +23500,16 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>G2M Slip (days)</t>
+          <t>Planned Quarter</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>g2m_slip_days</t>
+          <t>g2m_quarter</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -23425,25 +23528,25 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Business Value (12m run-rate)</t>
+          <t>G2M Slip (days)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>value_12m</t>
+          <t>g2m_slip_days</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111">
@@ -23453,16 +23556,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Business Value (12m run-rate)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>value_12m</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -23481,21 +23584,21 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>confidence</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G112" t="n">
@@ -23509,25 +23612,25 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Current Gate</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>current_gate</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Gates</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -23537,25 +23640,25 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Current Gate</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>current_gate</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Gates</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115">
@@ -23565,25 +23668,25 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>sponsor</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="116">
@@ -23593,21 +23696,21 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Next Review Date</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>next_review_date</t>
+          <t>sponsor</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G116" t="n">
@@ -23621,21 +23724,21 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Summary (participant-facing)</t>
+          <t>Next Review Date</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>next_review_date</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G117" t="n">
@@ -23645,25 +23748,20 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Discovery</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Summary (participant-facing)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -23673,11 +23771,6 @@
       </c>
       <c r="G118" t="n">
         <v>1</v>
-      </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="119">
@@ -23686,17 +23779,22 @@
           <t>Discovery</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Early-stage items: hypothesis, evidence, risks and the people involved. (Takes over the v4 Leadership content.)</t>
+        </is>
+      </c>
       <c r="C119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -23720,16 +23818,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -23753,16 +23851,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -23772,6 +23870,11 @@
       </c>
       <c r="G121" t="n">
         <v>1</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -23781,16 +23884,16 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Change Type</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>change_type</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -23809,16 +23912,16 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
+          <t>Change Type</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>hypothesis</t>
+          <t>change_type</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -23837,21 +23940,21 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Request Origin</t>
+          <t>Initiative Hypothesis (IF / THEN / RESULTING IN)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>request_origin</t>
+          <t>hypothesis</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -23865,16 +23968,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Customers Requesting (#)</t>
+          <t>Request Origin</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>customers_requesting</t>
+          <t>request_origin</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -23893,21 +23996,21 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Customers Requesting (#)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>customers_requesting</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G126" t="n">
@@ -23921,21 +24024,21 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Cost of Not Doing (strategic risk)</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>cost_of_not_doing</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G127" t="n">
@@ -23949,16 +24052,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Related / Overlaps With (Initiative IDs)</t>
+          <t>Cost of Not Doing (strategic risk)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>related_to</t>
+          <t>cost_of_not_doing</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -23977,16 +24080,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Dependencies / Blockers</t>
+          <t>Related / Overlaps With (Initiative IDs)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>dependencies_blockers</t>
+          <t>related_to</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -24005,16 +24108,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Business Value Type</t>
+          <t>Dependencies / Blockers</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>dependencies_blockers</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -24033,16 +24136,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Business Value Basis</t>
+          <t>Business Value Type</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>value_basis</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -24061,16 +24164,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Time to First Revenue (months)</t>
+          <t>Business Value Basis</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>time_to_first_revenue_months</t>
+          <t>value_basis</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -24089,16 +24192,16 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Primary KR (Metric Name)</t>
+          <t>Time to First Revenue (months)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>kr_metric</t>
+          <t>time_to_first_revenue_months</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -24117,16 +24220,16 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Primary KR Target Value</t>
+          <t>Primary KR (Metric Name)</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>kr_target</t>
+          <t>kr_metric</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -24145,21 +24248,21 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Artifacts (links)</t>
+          <t>Primary KR Target Value</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>artifacts</t>
+          <t>kr_target</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="G135" t="n">
@@ -24173,25 +24276,25 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Artifacts (links)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>artifacts</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Spec</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G136" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -24201,16 +24304,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Spec Status</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>spec_status</t>
+          <t>documents</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -24229,25 +24332,25 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Spec Status</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>product_manager</t>
+          <t>spec_status</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Spec</t>
         </is>
       </c>
       <c r="G138" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="139">
@@ -24257,16 +24360,16 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>designer</t>
+          <t>product_manager</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -24285,16 +24388,16 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>designer</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -24313,16 +24416,16 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Business Manager</t>
+          <t>Analyst</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>business_manager</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -24341,21 +24444,21 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>AI Draft (needs review)</t>
+          <t>Business Manager</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>ai_draft</t>
+          <t>business_manager</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="G142" t="n">
@@ -24365,39 +24468,29 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Timeline</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+          <t>Discovery</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>AI Draft (needs review)</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>ai_draft</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G143" t="n">
         <v>1</v>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="144">
@@ -24406,17 +24499,22 @@
           <t>Timeline</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>How long things take: phase start dates and durations. (The v4 Discovery content, renamed.)</t>
+        </is>
+      </c>
       <c r="C144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -24440,16 +24538,16 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -24473,16 +24571,16 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -24492,6 +24590,11 @@
       </c>
       <c r="G146" t="n">
         <v>1</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="147">
@@ -24501,25 +24604,25 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Days in Current Phase</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>days_in_phase</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G147" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -24529,25 +24632,25 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Days in Current Phase</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>days_in_phase</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149">
@@ -24557,16 +24660,16 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Start Discovery</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>start_discovery</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -24585,16 +24688,16 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Start Definition</t>
+          <t>Start Discovery</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>start_definition</t>
+          <t>start_discovery</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -24613,16 +24716,16 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Start Building</t>
+          <t>Start Definition</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>start_building</t>
+          <t>start_definition</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -24641,16 +24744,16 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Start Beta-Test</t>
+          <t>Start Building</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>start_beta</t>
+          <t>start_building</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -24669,16 +24772,16 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Start Experiment</t>
+          <t>Start Beta-Test</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>start_experiment</t>
+          <t>start_beta</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -24697,16 +24800,16 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Start Roll-Out</t>
+          <t>Start Experiment</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>start_rollout</t>
+          <t>start_experiment</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -24725,16 +24828,16 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>G2M Date (actual)</t>
+          <t>Start Roll-Out</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>g2m_date_actual</t>
+          <t>start_rollout</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -24753,25 +24856,25 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Discovery Time (days)</t>
+          <t>G2M Date (actual)</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>time_discovery_days</t>
+          <t>g2m_date_actual</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G156" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157">
@@ -24781,16 +24884,16 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Definition Time (days)</t>
+          <t>Discovery Time (days)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>time_definition_days</t>
+          <t>time_discovery_days</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -24809,16 +24912,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Building Time (days)</t>
+          <t>Definition Time (days)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>time_building_days</t>
+          <t>time_definition_days</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -24837,16 +24940,16 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Beta-Test Time (days)</t>
+          <t>Building Time (days)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>time_beta_days</t>
+          <t>time_building_days</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -24865,16 +24968,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Experiment Time (days)</t>
+          <t>Beta-Test Time (days)</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>time_experiment_days</t>
+          <t>time_beta_days</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -24893,16 +24996,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Roll-Out Time (days)</t>
+          <t>Experiment Time (days)</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>time_rollout_days</t>
+          <t>time_experiment_days</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -24921,16 +25024,16 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Time to Market (days)</t>
+          <t>Roll-Out Time (days)</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>time_to_market_days</t>
+          <t>time_rollout_days</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -24949,16 +25052,16 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Actual Build (weeks)</t>
+          <t>Time to Market (days)</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>actual_build_weeks</t>
+          <t>time_to_market_days</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -24977,16 +25080,16 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Build vs Estimate High (%)</t>
+          <t>Actual Build (weeks)</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>build_vs_estimate_high_pct</t>
+          <t>actual_build_weeks</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -25005,16 +25108,16 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Blocked Days</t>
+          <t>Build vs Estimate High (%)</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>blocked_days</t>
+          <t>build_vs_estimate_high_pct</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -25029,39 +25132,29 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>History</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Blocked Days</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>blocked_days</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G166" t="n">
-        <v>1</v>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="167">
@@ -25070,17 +25163,22 @@
           <t>History</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>What changed, when and by whom: audit-style columns and rank movement.</t>
+        </is>
+      </c>
       <c r="C167" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -25104,16 +25202,16 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -25137,25 +25235,30 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Planning Status</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>planning_status</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G169" t="n">
         <v>1</v>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="170">
@@ -25165,25 +25268,25 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Build Status</t>
+          <t>Planning Status</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>planning_status</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G170" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171">
@@ -25193,16 +25296,16 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Initiative Phase</t>
+          <t>Build Status</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>initiative_phase</t>
+          <t>status</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -25211,7 +25314,7 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172">
@@ -25221,16 +25324,16 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Initiative Phase</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>initiative_phase</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -25249,21 +25352,21 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G173" t="n">
@@ -25277,16 +25380,16 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Decided By</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>decided_by</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -25305,16 +25408,16 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Decision Date</t>
+          <t>Decided By</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>decision_date</t>
+          <t>decided_by</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -25333,21 +25436,21 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Status Changed At</t>
+          <t>Decision Date</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>status_changed_at</t>
+          <t>decision_date</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="G176" t="n">
@@ -25361,16 +25464,16 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Phase Changed At</t>
+          <t>Status Changed At</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>phase_changed_at</t>
+          <t>status_changed_at</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -25389,21 +25492,21 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>Phase Changed At</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>last_edited_at</t>
+          <t>phase_changed_at</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G178" t="n">
@@ -25417,21 +25520,21 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Last Edited By</t>
+          <t>Last Updated</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>last_edited_by</t>
+          <t>last_edited_at</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Trust</t>
+          <t>When</t>
         </is>
       </c>
       <c r="G179" t="n">
@@ -25445,16 +25548,16 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Created At</t>
+          <t>Last Edited By</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>last_edited_by</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -25473,16 +25576,16 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Created By</t>
+          <t>Created At</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -25501,16 +25604,16 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Created Via</t>
+          <t>Created By</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>created_via</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -25529,16 +25632,16 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Last Reviewed</t>
+          <t>Created Via</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>last_reviewed_at</t>
+          <t>created_via</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -25557,16 +25660,16 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Review Overdue</t>
+          <t>Last Reviewed</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>review_overdue</t>
+          <t>last_reviewed_at</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -25575,7 +25678,7 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185">
@@ -25585,16 +25688,16 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Item Age (days)</t>
+          <t>Review Overdue</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>item_age_days</t>
+          <t>review_overdue</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -25613,16 +25716,16 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Archived</t>
+          <t>Item Age (days)</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>item_age_days</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -25631,45 +25734,35 @@
         </is>
       </c>
       <c r="G186" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Cycle review</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Stack Rank</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>stack_rank</t>
+          <t>archived</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="G187" t="n">
         <v>1</v>
-      </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
       </c>
     </row>
     <row r="188">
@@ -25678,17 +25771,22 @@
           <t>Cycle review</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Planning-cycle triage: candidate pool, carry-over, deferrals and what was added after commit.</t>
+        </is>
+      </c>
       <c r="C188" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Initiative ID</t>
+          <t>Stack Rank</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>stack_rank</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -25712,16 +25810,16 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Initiative Name</t>
+          <t>Initiative ID</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>initiative_name</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -25745,16 +25843,16 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Home Project</t>
+          <t>Initiative Name</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>home_project</t>
+          <t>initiative_name</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -25764,6 +25862,11 @@
       </c>
       <c r="G190" t="n">
         <v>1</v>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
       </c>
     </row>
     <row r="191">
@@ -25773,16 +25876,16 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Initiative Status</t>
+          <t>Home Project</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>initiative_status</t>
+          <t>home_project</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -25801,25 +25904,25 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Initiative Status</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>cycle</t>
+          <t>initiative_status</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G192" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -25829,16 +25932,16 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Candidate Tag</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>candidate_tag</t>
+          <t>cycle</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -25857,16 +25960,16 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Deferred Count</t>
+          <t>Candidate Tag</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>deferred_count</t>
+          <t>candidate_tag</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -25885,16 +25988,16 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Deferral Reason</t>
+          <t>Deferred Count</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>deferral_reason</t>
+          <t>deferred_count</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -25913,16 +26016,16 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Added After Commit</t>
+          <t>Deferral Reason</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>added_after_commit</t>
+          <t>deferral_reason</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -25941,25 +26044,25 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Previous Rank</t>
+          <t>Added After Commit</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>previous_rank</t>
+          <t>added_after_commit</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="G197" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="198">
@@ -25969,21 +26072,21 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Effort (T-shirt)</t>
+          <t>Previous Rank</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>effort</t>
+          <t>previous_rank</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>What</t>
         </is>
       </c>
       <c r="G198" t="n">
@@ -25997,16 +26100,16 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Fit by Team</t>
+          <t>Effort (T-shirt)</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>fit_by_team</t>
+          <t>effort</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -26015,7 +26118,7 @@
         </is>
       </c>
       <c r="G199" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="200">
@@ -26025,16 +26128,16 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>MoSCoW</t>
+          <t>Fit by Team</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>moscow</t>
+          <t>fit_by_team</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -26043,7 +26146,7 @@
         </is>
       </c>
       <c r="G200" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="201">
@@ -26053,24 +26156,52 @@
         </is>
       </c>
       <c r="C201" t="n">
+        <v>14</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>MoSCoW</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>moscow</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="G201" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Cycle review</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
         <v>15</v>
       </c>
-      <c r="D201" t="inlineStr">
+      <c r="D202" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
+      <c r="E202" t="inlineStr">
         <is>
           <t>decision</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr">
+      <c r="F202" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="G201" t="n">
+      <c r="G202" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>